<commit_message>
Fix request display: filter invalid day values, fix migration logic
</commit_message>
<xml_diff>
--- a/api/backend/uploads/ibu_schedule.xlsx
+++ b/api/backend/uploads/ibu_schedule.xlsx
@@ -62029,7 +62029,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P85"/>
+  <dimension ref="A1:P87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -65722,7 +65722,92 @@
         </is>
       </c>
       <c r="M85" s="463" t="n">
-        <v>46182.78545583101</v>
+        <v>46182.78545583333</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>666e44a8-8e15-4ed4-9591-9eda49744c49</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>emp_1781043065177</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>day_off</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>["monday"]</t>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>AvailabilityRequestStatus.PENDING</t>
+        </is>
+      </c>
+      <c r="M86" s="463" t="n">
+        <v>46182.78808515046</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>a96dd354-5a74-48f9-a5ac-14b291a6f978</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>emp_1781043065177</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>day_off</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>["friday"]</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>AvailabilityRequestStatus.PENDING</t>
+        </is>
+      </c>
+      <c r="K87" t="inlineStr">
+        <is>
+          <t>Please approve.</t>
+        </is>
+      </c>
+      <c r="M87" s="463" t="n">
+        <v>46182.78831321914</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix ScheduleManager date filtering, add Excel file loading on startup
</commit_message>
<xml_diff>
--- a/api/backend/uploads/ibu_schedule.xlsx
+++ b/api/backend/uploads/ibu_schedule.xlsx
@@ -3146,7 +3146,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:V39"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -4754,7 +4754,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:V34"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -6253,7 +6253,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:V34"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -7695,7 +7695,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:V33"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -9041,7 +9041,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:V33"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -10483,7 +10483,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:V33"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -11951,7 +11951,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:V33"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -13285,7 +13285,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:U32"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="18.1640625" customWidth="1" min="2" max="2"/>
@@ -14644,7 +14644,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:U32"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -16006,7 +16006,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:U32"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -17352,7 +17352,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:U32"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -18722,7 +18722,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:V39"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -20305,7 +20305,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:U31"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -21595,7 +21595,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:U31"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -22936,7 +22936,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:U33"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="19.5" customWidth="1" min="2" max="2"/>
@@ -24396,7 +24396,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:U33"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -25729,7 +25729,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:U32"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -27004,7 +27004,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:Q31"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -28199,7 +28199,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:Q33"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -29501,7 +29501,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:Q33"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -30824,7 +30824,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:Q33"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -32125,7 +32125,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:Q33"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -33360,7 +33360,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:V39"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
@@ -34917,7 +34917,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:Q34"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -36181,7 +36181,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:Q34"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -37438,7 +37438,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:Q31"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -38515,7 +38515,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:Q31"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -39569,7 +39569,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:Q23"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -40621,7 +40621,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:Q24"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -41671,7 +41671,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:R24"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -42744,7 +42744,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:Q24"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -43795,7 +43795,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:Q23"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -44825,7 +44825,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:Q21"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -45767,7 +45767,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:V39"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -47274,7 +47274,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:P22"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -48257,7 +48257,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:Q21"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="17.5" customWidth="1" min="1" max="2"/>
     <col width="4.33203125" customWidth="1" min="3" max="3"/>
@@ -49174,7 +49174,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:Q23"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -50276,7 +50276,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:Q24"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="11.1640625" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -52152,7 +52152,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N91"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -65807,7 +65807,7 @@
         </is>
       </c>
       <c r="M87" s="463" t="n">
-        <v>46182.78831321914</v>
+        <v>46182.78831321759</v>
       </c>
     </row>
   </sheetData>
@@ -65823,7 +65823,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:V36"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -67333,7 +67333,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:AA36"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="35.5" customWidth="1" min="2" max="2"/>
@@ -68879,7 +68879,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:V35"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -70381,7 +70381,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:V36"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -71783,7 +71783,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:V33"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>

</xml_diff>

<commit_message>
Add employee preferences to locked shifts and scheduler
</commit_message>
<xml_diff>
--- a/api/backend/uploads/ibu_schedule.xlsx
+++ b/api/backend/uploads/ibu_schedule.xlsx
@@ -55,6 +55,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Events" sheetId="47" state="visible" r:id="rId47"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notifications" sheetId="48" state="visible" r:id="rId48"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Availability_Requests" sheetId="49" state="visible" r:id="rId49"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Schedule_2026_06_22" sheetId="50" state="visible" r:id="rId50"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191028" fullCalcOnLoad="1"/>
@@ -52151,7 +52152,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N91"/>
+  <dimension ref="A1:N94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -56600,7 +56601,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Test new employee</t>
+          <t>Manager Test</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -56651,7 +56652,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Test new employee</t>
+          <t>Manager Test</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -56702,7 +56703,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Test new employee</t>
+          <t>Manager Test</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -56753,7 +56754,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Test new employee</t>
+          <t>Manager Test</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -56804,7 +56805,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Test new employee</t>
+          <t>Manager Test</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -56839,6 +56840,164 @@
       <c r="N91" t="inlineStr">
         <is>
           <t>manager activities</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>locked_5b018a26-b30c-4096-8800-a408ae2e1ec5_2026-06-16</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>emp_1781043065177</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Normal worker Test</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>tuesday</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>desk</t>
+        </is>
+      </c>
+      <c r="I92" t="n">
+        <v>1</v>
+      </c>
+      <c r="J92" t="b">
+        <v>0</v>
+      </c>
+      <c r="L92" t="b">
+        <v>1</v>
+      </c>
+      <c r="M92" t="inlineStr">
+        <is>
+          <t>08:00 - 09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>locked_5f7d66fd-0994-478b-ad9b-e3a43d7c73fa_2026-06-15</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>emp_1781043065177</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Normal worker Test</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>monday</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>23:59</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>desk</t>
+        </is>
+      </c>
+      <c r="I93" t="n">
+        <v>23.98333333333333</v>
+      </c>
+      <c r="J93" t="b">
+        <v>0</v>
+      </c>
+      <c r="L93" t="b">
+        <v>1</v>
+      </c>
+      <c r="M93" t="inlineStr">
+        <is>
+          <t>Day Off</t>
+        </is>
+      </c>
+      <c r="N93" t="inlineStr">
+        <is>
+          <t>day off</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>locked_18c13503-ccac-4829-bf54-b3a5a943ead5_2026-06-17</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>emp_1781043065177</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Normal worker Test</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>wednesday</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>desk</t>
+        </is>
+      </c>
+      <c r="I94" t="n">
+        <v>5</v>
+      </c>
+      <c r="J94" t="b">
+        <v>0</v>
+      </c>
+      <c r="L94" t="b">
+        <v>1</v>
+      </c>
+      <c r="M94" t="inlineStr">
+        <is>
+          <t>12:00 - 17:00</t>
         </is>
       </c>
     </row>
@@ -57027,7 +57186,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F178"/>
+  <dimension ref="A1:F186"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -62016,6 +62175,230 @@
       </c>
       <c r="F178" t="b">
         <v>0</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>39b64f24-d424-43b1-a3da-ba79f60bd6c1</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>emp_1781043065177</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>NotificationType.AVAILABILITY_REJECTED</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>Your day_off request (2026-06-09 to 2026-06-15) was not approved. Reason: Sorry.</t>
+        </is>
+      </c>
+      <c r="E179" s="463" t="n">
+        <v>46182.80566836806</v>
+      </c>
+      <c r="F179" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>17c9abca-bd06-444e-a589-e58ff4fe501a</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>emp_1781043065177</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>NotificationType.AVAILABILITY_APPROVED</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>Your availability request (2026-06-10 to 2026-06-26) has been approved. Manager note: ok</t>
+        </is>
+      </c>
+      <c r="E180" s="463" t="n">
+        <v>46182.80733979167</v>
+      </c>
+      <c r="F180" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>0ad2dc2f-1cb0-48dc-a53d-cb5261bd30f2</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>emp_1781043065177</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>NotificationType.AVAILABILITY_APPROVED</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>Your day_off request (2026-06-12 to 2026-06-12) has been approved.</t>
+        </is>
+      </c>
+      <c r="E181" s="463" t="n">
+        <v>46182.80738758102</v>
+      </c>
+      <c r="F181" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>ca9ce35d-8efc-474e-815a-d4c52b92aeda</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>emp_1781043065177</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>NotificationType.AVAILABILITY_APPROVED</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>Your day_off request (2026-06-15 to 2026-06-22) has been approved.</t>
+        </is>
+      </c>
+      <c r="E182" s="463" t="n">
+        <v>46182.80756181713</v>
+      </c>
+      <c r="F182" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>4c87d280-dd11-46be-9688-47f45a7bc455</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>emp_1781043065177</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>NotificationType.AVAILABILITY_APPROVED</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>Your day_off request (2026-06-18 to 2026-06-18) has been approved.</t>
+        </is>
+      </c>
+      <c r="E183" s="463" t="n">
+        <v>46182.8075971412</v>
+      </c>
+      <c r="F183" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>2aca14e0-49e8-42da-8bfa-e663c23c9451</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>emp_1781043065177</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>NotificationType.AVAILABILITY_APPROVED</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>Your day_off request (2026-06-15 to 2026-06-22) has been approved.</t>
+        </is>
+      </c>
+      <c r="E184" s="463" t="n">
+        <v>46182.80764542824</v>
+      </c>
+      <c r="F184" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>40537a05-b02f-4572-b718-62d63485ee18</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>emp_1781043065177</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>NotificationType.AVAILABILITY_APPROVED</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>Your availability request (2026-06-16 to 2026-06-26) has been approved.</t>
+        </is>
+      </c>
+      <c r="E185" s="463" t="n">
+        <v>46182.80769424768</v>
+      </c>
+      <c r="F185" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>5de7943e-6cdf-4318-8d34-38197ae00a82</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>emp_1781043065177</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>NotificationType.AVAILABILITY_REJECTED</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>Your day_off request (2026-06-23 to 2026-06-23) was not approved. Reason: s</t>
+        </is>
+      </c>
+      <c r="E186" s="463" t="n">
+        <v>46182.80940947917</v>
+      </c>
+      <c r="F186" t="b">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -62029,7 +62412,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P87"/>
+  <dimension ref="A1:P91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -65673,12 +66056,20 @@
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>AvailabilityRequestStatus.PENDING</t>
+          <t>AvailabilityRequestStatus.REJECTED</t>
+        </is>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>Sorry.</t>
         </is>
       </c>
       <c r="M84" s="463" t="n">
         <v>46182.78526831019</v>
       </c>
+      <c r="N84" s="463" t="n">
+        <v>46182.80566619213</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -65713,7 +66104,12 @@
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>AvailabilityRequestStatus.PENDING</t>
+          <t>AvailabilityRequestStatus.REJECTED</t>
+        </is>
+      </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>s</t>
         </is>
       </c>
       <c r="K85" t="inlineStr">
@@ -65724,6 +66120,9 @@
       <c r="M85" s="463" t="n">
         <v>46182.78545583333</v>
       </c>
+      <c r="N85" s="463" t="n">
+        <v>46182.80940729166</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -65758,12 +66157,23 @@
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>AvailabilityRequestStatus.PENDING</t>
+          <t>AvailabilityRequestStatus.APPROVED</t>
         </is>
       </c>
       <c r="M86" s="463" t="n">
         <v>46182.78808515046</v>
       </c>
+      <c r="N86" s="463" t="n">
+        <v>46182.80754699074</v>
+      </c>
+      <c r="O86" t="inlineStr">
+        <is>
+          <t>emp_1780946033840</t>
+        </is>
+      </c>
+      <c r="P86" s="463" t="n">
+        <v>46182.80754699074</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -65798,7 +66208,7 @@
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>AvailabilityRequestStatus.PENDING</t>
+          <t>AvailabilityRequestStatus.APPROVED</t>
         </is>
       </c>
       <c r="K87" t="inlineStr">
@@ -65808,6 +66218,266 @@
       </c>
       <c r="M87" s="463" t="n">
         <v>46182.78831321759</v>
+      </c>
+      <c r="N87" s="463" t="n">
+        <v>46182.80759497685</v>
+      </c>
+      <c r="O87" t="inlineStr">
+        <is>
+          <t>emp_1780946033840</t>
+        </is>
+      </c>
+      <c r="P87" s="463" t="n">
+        <v>46182.80759497685</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>5f7d66fd-0994-478b-ad9b-e3a43d7c73fa</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>emp_1781043065177</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>day_off</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>["monday"]</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>AvailabilityRequestStatus.APPROVED</t>
+        </is>
+      </c>
+      <c r="K88" t="inlineStr">
+        <is>
+          <t>Approve boss.</t>
+        </is>
+      </c>
+      <c r="M88" s="463" t="n">
+        <v>46182.80669766204</v>
+      </c>
+      <c r="N88" s="463" t="n">
+        <v>46182.80763089121</v>
+      </c>
+      <c r="O88" t="inlineStr">
+        <is>
+          <t>emp_1780946033840</t>
+        </is>
+      </c>
+      <c r="P88" s="463" t="n">
+        <v>46182.80763089121</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>5b018a26-b30c-4096-8800-a408ae2e1ec5</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>emp_1781043065177</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>availability</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>["tuesday"]</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>AvailabilityRequestStatus.APPROVED</t>
+        </is>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="K89" t="inlineStr">
+        <is>
+          <t>Approve boss.</t>
+        </is>
+      </c>
+      <c r="M89" s="463" t="n">
+        <v>46182.80669996528</v>
+      </c>
+      <c r="N89" s="463" t="n">
+        <v>46182.80732481481</v>
+      </c>
+      <c r="O89" t="inlineStr">
+        <is>
+          <t>emp_1780946033840</t>
+        </is>
+      </c>
+      <c r="P89" s="463" t="n">
+        <v>46182.80732481481</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>18c13503-ccac-4829-bf54-b3a5a943ead5</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>emp_1781043065177</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>availability</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>["wednesday"]</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>AvailabilityRequestStatus.APPROVED</t>
+        </is>
+      </c>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>Approve boss.</t>
+        </is>
+      </c>
+      <c r="M90" s="463" t="n">
+        <v>46182.80670422454</v>
+      </c>
+      <c r="N90" s="463" t="n">
+        <v>46182.80767947916</v>
+      </c>
+      <c r="O90" t="inlineStr">
+        <is>
+          <t>emp_1780946033840</t>
+        </is>
+      </c>
+      <c r="P90" s="463" t="n">
+        <v>46182.80767947916</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>a5f2092e-9afe-45e5-89f2-7b90194ac3b4</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>emp_1781043065177</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>day_off</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>["saturday"]</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>AvailabilityRequestStatus.APPROVED</t>
+        </is>
+      </c>
+      <c r="K91" t="inlineStr">
+        <is>
+          <t>Have an external event.</t>
+        </is>
+      </c>
+      <c r="M91" s="463" t="n">
+        <v>46182.80686585648</v>
+      </c>
+      <c r="N91" s="463" t="n">
+        <v>46182.80738541667</v>
+      </c>
+      <c r="O91" t="inlineStr">
+        <is>
+          <t>emp_1780946033840</t>
+        </is>
+      </c>
+      <c r="P91" s="463" t="n">
+        <v>46182.80738541667</v>
       </c>
     </row>
   </sheetData>
@@ -67322,6 +67992,266 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet50.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="15" customWidth="1" min="12" max="12"/>
+    <col width="15" customWidth="1" min="13" max="13"/>
+    <col width="15" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="460" t="inlineStr">
+        <is>
+          <t>Shift_ID</t>
+        </is>
+      </c>
+      <c r="B1" s="460" t="inlineStr">
+        <is>
+          <t>Employee_ID</t>
+        </is>
+      </c>
+      <c r="C1" s="460" t="inlineStr">
+        <is>
+          <t>Employee_Name</t>
+        </is>
+      </c>
+      <c r="D1" s="460" t="inlineStr">
+        <is>
+          <t>Day</t>
+        </is>
+      </c>
+      <c r="E1" s="460" t="inlineStr">
+        <is>
+          <t>Start_Time</t>
+        </is>
+      </c>
+      <c r="F1" s="460" t="inlineStr">
+        <is>
+          <t>End_Time</t>
+        </is>
+      </c>
+      <c r="G1" s="460" t="inlineStr">
+        <is>
+          <t>Job_Type</t>
+        </is>
+      </c>
+      <c r="H1" s="460" t="inlineStr">
+        <is>
+          <t>Floor</t>
+        </is>
+      </c>
+      <c r="I1" s="460" t="inlineStr">
+        <is>
+          <t>Hours</t>
+        </is>
+      </c>
+      <c r="J1" s="460" t="inlineStr">
+        <is>
+          <t>Is_Event</t>
+        </is>
+      </c>
+      <c r="K1" s="460" t="inlineStr">
+        <is>
+          <t>Event_Name</t>
+        </is>
+      </c>
+      <c r="L1" s="460" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+      <c r="M1" s="460" t="inlineStr">
+        <is>
+          <t>Locked_Avail_Type</t>
+        </is>
+      </c>
+      <c r="N1" s="460" t="inlineStr">
+        <is>
+          <t>Location</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>locked_5b018a26-b30c-4096-8800-a408ae2e1ec5_2026-06-23</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>emp_1781043065177</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Normal worker Test</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>tuesday</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>desk</t>
+        </is>
+      </c>
+      <c r="I2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J2" t="b">
+        <v>0</v>
+      </c>
+      <c r="L2" t="b">
+        <v>1</v>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>08:00 - 09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>locked_5f7d66fd-0994-478b-ad9b-e3a43d7c73fa_2026-06-22</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>emp_1781043065177</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Normal worker Test</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>monday</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>23:59</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>desk</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>23.98333333333333</v>
+      </c>
+      <c r="J3" t="b">
+        <v>0</v>
+      </c>
+      <c r="L3" t="b">
+        <v>1</v>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Day Off</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>day off</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>locked_18c13503-ccac-4829-bf54-b3a5a943ead5_2026-06-24</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>emp_1781043065177</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Normal worker Test</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>wednesday</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>desk</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>5</v>
+      </c>
+      <c r="J4" t="b">
+        <v>0</v>
+      </c>
+      <c r="L4" t="b">
+        <v>1</v>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>12:00 - 17:00</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Fix pending requests panel to only show pending status
</commit_message>
<xml_diff>
--- a/api/backend/uploads/ibu_schedule.xlsx
+++ b/api/backend/uploads/ibu_schedule.xlsx
@@ -3147,7 +3147,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:V39"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -4755,7 +4755,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:V34"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -6254,7 +6254,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:V34"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -7696,7 +7696,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:V33"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -9042,7 +9042,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:V33"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -10484,7 +10484,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:V33"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -11952,7 +11952,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:V33"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -13286,7 +13286,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:U32"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="18.1640625" customWidth="1" min="2" max="2"/>
@@ -14645,7 +14645,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:U32"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -16007,7 +16007,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:U32"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -17353,7 +17353,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:U32"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -18723,7 +18723,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:V39"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -20306,7 +20306,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:U31"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -21596,7 +21596,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:U31"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -22937,7 +22937,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:U33"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="19.5" customWidth="1" min="2" max="2"/>
@@ -24397,7 +24397,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:U33"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -25730,7 +25730,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:U32"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -27005,7 +27005,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:Q31"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -28200,7 +28200,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:Q33"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -29502,7 +29502,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:Q33"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -30825,7 +30825,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:Q33"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -32126,7 +32126,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:Q33"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -33361,7 +33361,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:V39"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
@@ -34918,7 +34918,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:Q34"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -36182,7 +36182,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:Q34"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -37439,7 +37439,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:Q31"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -38516,7 +38516,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:Q31"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -39570,7 +39570,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:Q23"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -40622,7 +40622,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:Q24"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -41672,7 +41672,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:R24"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -42745,7 +42745,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:Q24"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -43796,7 +43796,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:Q23"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -44826,7 +44826,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:Q21"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -45768,7 +45768,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:V39"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -47275,7 +47275,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:P22"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -48258,7 +48258,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:Q21"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="17.5" customWidth="1" min="1" max="2"/>
     <col width="4.33203125" customWidth="1" min="3" max="3"/>
@@ -49175,7 +49175,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:Q23"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -50277,7 +50277,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:Q24"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="11.1640625" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -52153,7 +52153,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N94"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -62412,7 +62412,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P91"/>
+  <dimension ref="A1:P93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -66478,6 +66478,87 @@
       </c>
       <c r="P91" s="463" t="n">
         <v>46182.80738541667</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>8b88681b-4d8c-4765-a0ed-34f658bc02ef</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>emp_1781047684821</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>day_off</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>["monday"]</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>AvailabilityRequestStatus.PENDING</t>
+        </is>
+      </c>
+      <c r="M92" s="463" t="n">
+        <v>46182.81649952546</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>72d4bfe1-dd9b-402e-a50e-b348cf60a70f</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>emp_1781047684821</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>day_off</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>["thursday"]</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>AvailabilityRequestStatus.PENDING</t>
+        </is>
+      </c>
+      <c r="K93" t="inlineStr"/>
+      <c r="M93" s="463" t="n">
+        <v>46182.81661243009</v>
       </c>
     </row>
   </sheetData>
@@ -66493,7 +66574,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:V36"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -68002,7 +68083,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -68263,7 +68344,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:AA36"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="35.5" customWidth="1" min="2" max="2"/>
@@ -69809,7 +69890,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:V35"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -71311,7 +71392,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:V36"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -72713,7 +72794,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:V33"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>

</xml_diff>

<commit_message>
Add persistent employee preferences with save button
</commit_message>
<xml_diff>
--- a/api/backend/uploads/ibu_schedule.xlsx
+++ b/api/backend/uploads/ibu_schedule.xlsx
@@ -62509,7 +62509,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P93"/>
+  <dimension ref="A1:P95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -66674,6 +66674,102 @@
       </c>
       <c r="N93" s="463" t="n">
         <v>46182.81902396991</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>d4aaa49b-72e3-4e1c-9db0-c68ab1ca966f</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>emp_1781047684821</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>day_off</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>["monday"]</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>AvailabilityRequestStatus.PENDING</t>
+        </is>
+      </c>
+      <c r="M94" s="463" t="n">
+        <v>46182.82825238426</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>365e0a5b-8b06-4ca7-a1c8-92c4eb3bd061</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>emp_1781047684821</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>availability</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>["tuesday"]</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>AvailabilityRequestStatus.PENDING</t>
+        </is>
+      </c>
+      <c r="K95" t="inlineStr"/>
+      <c r="L95" t="inlineStr">
+        <is>
+          <t>{'ground_floor': 10, 'second_floor': 9, 'sixth_floor': 8, 'call_center': 7, 'event': 6}</t>
+        </is>
+      </c>
+      <c r="M95" s="463" t="n">
+        <v>46182.82825483126</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix progress bar not showing during auto-generate
</commit_message>
<xml_diff>
--- a/api/backend/uploads/ibu_schedule.xlsx
+++ b/api/backend/uploads/ibu_schedule.xlsx
@@ -3148,7 +3148,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:V39"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -4756,7 +4756,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:V34"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -6255,7 +6255,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:V34"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -7697,7 +7697,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:V33"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -9043,7 +9043,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:V33"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -10485,7 +10485,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:V33"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -11953,7 +11953,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:V33"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -13287,7 +13287,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:U32"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="18.1640625" customWidth="1" min="2" max="2"/>
@@ -14646,7 +14646,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:U32"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -16008,7 +16008,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:U32"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -17354,7 +17354,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:U32"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -18724,7 +18724,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:V39"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -20307,7 +20307,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:U31"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -21597,7 +21597,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:U31"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -22938,7 +22938,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:U33"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="19.5" customWidth="1" min="2" max="2"/>
@@ -24398,7 +24398,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:U33"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -25731,7 +25731,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:U32"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -27006,7 +27006,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:Q31"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -28201,7 +28201,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:Q33"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -29503,7 +29503,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:Q33"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -30826,7 +30826,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:Q33"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -32127,7 +32127,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:Q33"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -33362,7 +33362,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:V39"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
@@ -34919,7 +34919,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:Q34"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -36183,7 +36183,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:Q34"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -37440,7 +37440,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:Q31"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -38517,7 +38517,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:Q31"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -39571,7 +39571,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:Q23"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -40623,7 +40623,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:Q24"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -41673,7 +41673,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:R24"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -42746,7 +42746,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:Q24"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -43797,7 +43797,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:Q23"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -44827,7 +44827,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:Q21"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -45769,7 +45769,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:V39"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -47276,7 +47276,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:P22"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -48259,7 +48259,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:Q21"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="17.5" customWidth="1" min="1" max="2"/>
     <col width="4.33203125" customWidth="1" min="3" max="3"/>
@@ -49176,7 +49176,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:Q23"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -50278,7 +50278,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:Q24"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="11.1640625" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -52154,7 +52154,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N97"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -67189,7 +67189,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:V36"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -68697,8 +68697,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N105"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:N102"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -68791,7 +68791,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>434699a2-bd7e-4612-b04a-a157140337c5</t>
+          <t>ddf6b6c6-8759-4a7f-8b74-c04db71a445d</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -68842,7 +68842,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>94d92005-1bb1-4387-b916-73fbc9e45dd1</t>
+          <t>c53aec0d-5261-44cb-8063-8b78aa585c65</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -68893,7 +68893,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0fc91c7a-ed91-44cb-859e-d5b995a8feab</t>
+          <t>cbfc45a5-2262-43ac-a81d-aac7536af2f0</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -68944,7 +68944,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ccc48e3a-ad0a-4d90-b991-8b413aa47611</t>
+          <t>8d04c852-7d73-4204-ab7f-177774eefcac</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -68995,7 +68995,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>5ec20b6c-f30a-459b-a87d-4f4ef4115298</t>
+          <t>9de14841-c639-4b19-b00a-66a5dac4deb3</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -69046,7 +69046,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0585cc11-0d5c-441a-9d4c-5d6e34c1768c</t>
+          <t>8357d5f9-b465-4b9f-bbc4-79bc9bc7a5ed</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -69097,7 +69097,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>bb19bcae-852c-4064-bf84-cb8c50673d33</t>
+          <t>428a3d17-8f63-4aea-b1ad-99b3c8f69afd</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -69148,7 +69148,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>729458fd-3df9-4a7b-a257-8c5f96849dde</t>
+          <t>19a431be-cd64-4460-ba71-b783c1ab010d</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -69199,7 +69199,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>4335801f-3803-4f8f-8c1a-0250b9f93d4f</t>
+          <t>bd83aa05-e768-4d79-a664-74726d0e3dd0</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -69250,7 +69250,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>6f661118-a802-42fe-b5ee-b5c9ed49c84d</t>
+          <t>d77bfe77-dfa0-4ce4-8b2c-4992807224ad</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -69301,17 +69301,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>9630588b-0fb0-44af-9b68-044cb6a59ffa</t>
+          <t>c42d9d26-3276-4072-9cc6-23eb03a98da0</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>emp_1781047684821</t>
+          <t>emp_003</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Test New Worker</t>
+          <t>Nahim</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -69352,17 +69352,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>3d812c92-0999-4148-8fb6-3513adae2e29</t>
+          <t>31c11537-631f-4949-b110-56f5ffcba1dc</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>emp_1781047684821</t>
+          <t>emp_003</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Test New Worker</t>
+          <t>Nahim</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -69403,17 +69403,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>119004a5-0a73-4ec2-a26c-6cb6445141a5</t>
+          <t>f560f98f-7bb7-4fef-a0b9-fb27941cc934</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>emp_1781047684821</t>
+          <t>emp_007</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Test New Worker</t>
+          <t>Viviana</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -69454,17 +69454,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>67ebf2cb-a7f1-4c8c-b855-0f3d8c99a7aa</t>
+          <t>82d4ce62-f524-47d4-9f69-779b6b6aa6fe</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>emp_003</t>
+          <t>emp_009</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Nahim</t>
+          <t>Meg</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -69505,7 +69505,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>29aab983-5055-4671-92e3-1dc15c59483c</t>
+          <t>a8a87db0-eee2-4453-aac6-25014a442431</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -69556,7 +69556,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>460b4933-74d6-4dc4-a398-3fac1cb4bddd</t>
+          <t>5bb297f8-5e30-47c0-8b2e-29bdd6a01fbb</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -69607,7 +69607,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>c8509bb1-532e-4b59-a1f1-a1c30c1f3ab3</t>
+          <t>87396322-661a-45dd-ad4e-b9f7b8371e0c</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -69658,7 +69658,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>37602f2b-b18c-493f-bb5b-f722784bf5cc</t>
+          <t>7b45cf91-2cf0-4621-b000-78b4d2e37129</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -69709,7 +69709,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>af11ef2e-419b-4782-bb15-e77de01f79e5</t>
+          <t>655ad4b3-b52c-40cf-b4ef-d3f7ee419944</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -69760,17 +69760,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>4a0cb408-16bc-48fe-986a-6c4f58e19111</t>
+          <t>521f28b6-100f-48b3-8614-b0c185d95ff7</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>emp_007</t>
+          <t>emp_015</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Viviana</t>
+          <t>Itohan</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -69811,17 +69811,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>080b1ef8-4d29-46c0-b16a-241dbe79fe78</t>
+          <t>bd52963d-a32b-4975-9362-3c391716b35b</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>emp_1781047684821</t>
+          <t>emp_012</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Test New Worker</t>
+          <t>Arfa C</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -69862,17 +69862,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>3afa2a8c-7f53-403b-982c-84ba701d6fb3</t>
+          <t>f40fec7f-b9bc-4d20-9267-fda12c7c17aa</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>emp_009</t>
+          <t>emp_003</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Meg</t>
+          <t>Nahim</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -69913,17 +69913,17 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>98edec9b-d550-419c-b5f8-cec15a16e057</t>
+          <t>fef8cf86-6271-42c4-b4bc-46e0ad1f7fa9</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>emp_012</t>
+          <t>emp_007</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Arfa C</t>
+          <t>Viviana</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -69964,17 +69964,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>07ef5b23-b0f3-4128-95dc-9c07f91a4e5c</t>
+          <t>9fc903d4-bc15-4ca2-a421-e7034794ef60</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>emp_003</t>
+          <t>emp_014</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Nahim</t>
+          <t>Sagar C</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -70015,7 +70015,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>8bf34bf2-231d-49c9-aaae-18f55440718b</t>
+          <t>93f9ce83-50bc-4a48-ba7e-deccd721e240</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -70066,17 +70066,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>9072d2b7-cb02-46e4-986c-4107d6aa58ef</t>
+          <t>9239e818-4083-4d34-93d6-2b78dea8592c</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>emp_1781047684821</t>
+          <t>emp_008</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Test New Worker</t>
+          <t>Anastasia</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -70117,17 +70117,17 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>f8a4b940-e36a-453d-a6d9-54d14d196b1d</t>
+          <t>04c52363-1a46-4168-9337-7714659e1199</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>emp_1781047684821</t>
+          <t>emp_009</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Test New Worker</t>
+          <t>Meg</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -70168,7 +70168,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>736343a0-1ec9-4d9b-b19b-ac69c57a5ce1</t>
+          <t>1ab12f6c-3d25-4bd7-982b-340de0cd8b20</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -70219,17 +70219,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>6e7581b9-655f-4d3c-8a5d-a7df19a6ec94</t>
+          <t>1eb53ccb-eeeb-48ed-8c88-e277bdf795b3</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>emp_015</t>
+          <t>emp_004</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Itohan</t>
+          <t>Pablo</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -70270,17 +70270,17 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>a6f96abc-34e1-468e-865b-465768c11b08</t>
+          <t>2290f47f-fa94-4397-88b5-908959f44c87</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>emp_004</t>
+          <t>emp_015</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Pablo</t>
+          <t>Itohan</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -70321,17 +70321,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>5e36efdf-6d6c-40e0-a8c7-c7b0389b3f51</t>
+          <t>3ce1b20b-d65d-4c5b-a7c8-f9db5357f19b</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>emp_007</t>
+          <t>emp_1781047684821</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Viviana</t>
+          <t>Test New Worker</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -70372,17 +70372,17 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>769b862b-3c56-478a-b15a-35a4b0795286</t>
+          <t>57510fef-b553-428a-b2ab-c528d2c4a175</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>emp_012</t>
+          <t>emp_1781047684821</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Arfa C</t>
+          <t>Test New Worker</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -70423,17 +70423,17 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>d805ea2c-0ea3-4a67-b2a6-c563d7438487</t>
+          <t>a5dea3db-bfed-422a-8432-909dcb259fcc</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>emp_014</t>
+          <t>emp_1781047684821</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Sagar C</t>
+          <t>Test New Worker</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -70474,17 +70474,17 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>9ff29f2f-a351-4806-9b98-c6fd0fb93ad0</t>
+          <t>e979c654-b81a-414c-8e55-cb1cbf31a196</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>emp_009</t>
+          <t>emp_012</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Meg</t>
+          <t>Arfa C</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -70525,17 +70525,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>b7b42901-d788-44ad-a6db-6b033286fd87</t>
+          <t>413fec59-af83-4d29-bf95-816b2cfcffff</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>emp_008</t>
+          <t>emp_011</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Anastasia</t>
+          <t>Priyanka</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -70576,17 +70576,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>1fdbdf1c-5c72-429d-b8c5-e366d1964910</t>
+          <t>07021605-7a1b-45d4-8794-d592ab95c3c5</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>emp_011</t>
+          <t>emp_013</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Priyanka</t>
+          <t>Taran C</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -70627,17 +70627,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>d02bf0d9-7d23-46cb-bc90-179d945d28d4</t>
+          <t>4f64639c-5421-418f-8bb1-157db36d2b06</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>emp_013</t>
+          <t>emp_016</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Taran C</t>
+          <t>Arnob</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -70678,17 +70678,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>028159b9-eb5c-473b-a466-c36cc58543da</t>
+          <t>bd428c34-fbd0-489f-8d61-151a1023b2f7</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>emp_006</t>
+          <t>emp_003</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Mickaela  C</t>
+          <t>Nahim</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -70729,17 +70729,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>626091ac-2d7c-468e-9359-5d7e0bdcc758</t>
+          <t>a5cc59dc-f7a7-4f67-a6df-a1a8639eb69b</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>emp_015</t>
+          <t>emp_004</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Itohan</t>
+          <t>Pablo</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -70780,17 +70780,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>ab03328b-3c89-4ac8-82ef-80fb4f45eaaa</t>
+          <t>fb498cd6-c381-4013-844e-8d7e14f6fcf3</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>emp_004</t>
+          <t>emp_007</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Pablo</t>
+          <t>Viviana</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -70831,17 +70831,17 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>fc06e404-fcbc-45ac-ba4b-f343620dd56f</t>
+          <t>4f28a7be-cd9f-407e-b0ae-da819eb6a2f1</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>emp_007</t>
+          <t>emp_1781047684821</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Viviana</t>
+          <t>Test New Worker</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -70882,17 +70882,17 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>9c679333-c034-4d4b-985f-0b9b7a64e414</t>
+          <t>20f08772-6031-49ab-9b47-b13cd7f88ced</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>emp_012</t>
+          <t>emp_003</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Arfa C</t>
+          <t>Nahim</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -70933,17 +70933,17 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>44b8007f-6205-4fbb-8905-d53dbe723f3f</t>
+          <t>e14f3ac8-8bb9-4f89-a75d-cbc4ea395d0f</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>emp_014</t>
+          <t>emp_005</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Sagar C</t>
+          <t>Kavya C</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -70984,17 +70984,17 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>36c24220-9de5-4b25-bd3c-a8f8e4ea9a4c</t>
+          <t>24eb5a97-ea2a-4f9b-b7ac-208c20f578ae</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>emp_005</t>
+          <t>emp_007</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Kavya C</t>
+          <t>Viviana</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -71035,17 +71035,17 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>cdd1dd87-87bb-49d6-b4ac-62dc22fc02c2</t>
+          <t>54279a42-4f83-4eed-b383-6c0f834141ee</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>emp_016</t>
+          <t>emp_008</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Arnob</t>
+          <t>Anastasia</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -71086,17 +71086,17 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>ff3eb288-2a38-4437-9793-587ff0e1534d</t>
+          <t>28bf11cd-57ea-40a4-a4f9-86b8d958b763</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>emp_008</t>
+          <t>emp_1781047684821</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Anastasia</t>
+          <t>Test New Worker</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -71137,17 +71137,17 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>c492bdad-3769-4e1a-8f35-bedda0dbaf07</t>
+          <t>b32be596-e7f5-4c73-b7a0-6cb27165d849</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>emp_011</t>
+          <t>emp_1781047684821</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Priyanka</t>
+          <t>Test New Worker</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -71188,17 +71188,17 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>25583c40-564d-4658-b08c-02f648df9627</t>
+          <t>bf3a77c1-494d-4903-b11c-3ee6f237ac64</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>emp_003</t>
+          <t>emp_006</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Nahim</t>
+          <t>Mickaela  C</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -71239,7 +71239,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2adf35df-a50f-4550-8e21-83b0e3cbe125</t>
+          <t>19d74442-de67-47ec-8353-41f01f480ea1</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -71290,7 +71290,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>f44622ee-7f70-43fc-b683-ff5b2ec720cb</t>
+          <t>246f0e9a-d44f-43a2-acc7-02fbd0081dcf</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -71341,17 +71341,17 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>5de01ee5-f963-418a-84ef-a31e2ddca243</t>
+          <t>724ed3f8-698a-4cb8-8f2d-b1b3307559eb</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>emp_007</t>
+          <t>emp_005</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Viviana</t>
+          <t>Kavya C</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -71392,17 +71392,17 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>871b1679-0a20-40ea-8c03-c622e73c060d</t>
+          <t>c723f8c4-beaf-46b7-9b8c-af4704e6c4f4</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>emp_013</t>
+          <t>emp_011</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Taran C</t>
+          <t>Priyanka</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -71443,17 +71443,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>933b5034-c721-4261-91bc-4f4625649423</t>
+          <t>ccca2b37-242a-4f98-b404-a656a5b366df</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>emp_016</t>
+          <t>emp_013</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Arnob</t>
+          <t>Taran C</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -71494,17 +71494,17 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>ec6e9428-d651-4b80-9064-6bb6c9e58ea0</t>
+          <t>03e5df37-d433-4e7c-8b80-a58440f3f300</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>emp_009</t>
+          <t>emp_016</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Meg</t>
+          <t>Arnob</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -71545,17 +71545,17 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>89d9321a-704a-4417-9b3e-ae39839f2f6b</t>
+          <t>e2520c08-ff5e-4f43-b847-68e744f3afda</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>emp_008</t>
+          <t>emp_009</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Anastasia</t>
+          <t>Meg</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -71596,7 +71596,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>73f952b1-0f3e-426b-830c-fa9574fd60b5</t>
+          <t>b5663478-c85a-4e73-b0b2-c84e00d4d1bb</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -71647,7 +71647,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>4f8256db-c73b-4504-a579-c191a770a2ec</t>
+          <t>d66bf4ab-5075-4d36-852a-341a583d3e3f</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -71698,7 +71698,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>a7d21dc6-9dde-435f-87b7-70bd7943a158</t>
+          <t>e688220d-3a04-4062-8f41-7e84f1f25fa8</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -71749,7 +71749,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>9dd1458f-1812-4a8b-8b0b-afd4e5770925</t>
+          <t>862a3073-d1f5-419e-9ac2-f6f2e5b6fd60</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -71800,17 +71800,17 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>7e55b609-29a1-4775-a15c-77dab0e3649a</t>
+          <t>60055902-d777-47bf-9533-3f5b1fbaaa94</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>emp_007</t>
+          <t>emp_013</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Viviana</t>
+          <t>Taran C</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -71820,17 +71820,17 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
           <t>12:00</t>
         </is>
       </c>
-      <c r="F61" t="inlineStr">
-        <is>
-          <t>16:00</t>
-        </is>
-      </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>second_floor</t>
+          <t>call_center</t>
         </is>
       </c>
       <c r="I61" t="n">
@@ -71844,14 +71844,14 @@
       </c>
       <c r="N61" t="inlineStr">
         <is>
-          <t>2nd floor</t>
+          <t>call center</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>35fd36f0-d8cf-44b9-8eec-7ec753945df1</t>
+          <t>dd291705-2dfb-438c-a2fe-a48d1ace8664</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -71871,12 +71871,12 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>08:00</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
@@ -71902,7 +71902,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>6e3d9091-1e97-441f-a441-c8aad899dbac</t>
+          <t>ca31c341-2358-4210-ba23-3d2cb3c2e4a0</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -71922,12 +71922,12 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
@@ -71953,17 +71953,17 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>61c29151-c5ee-448f-81ba-dd373b9aa52d</t>
+          <t>21b5c4d1-46db-4119-a8ab-476365be56be</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>emp_013</t>
+          <t>emp_011</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Taran C</t>
+          <t>Priyanka</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -71973,17 +71973,17 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>08:00</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>call_center</t>
+          <t>ground_floor</t>
         </is>
       </c>
       <c r="I64" t="n">
@@ -71997,14 +71997,14 @@
       </c>
       <c r="N64" t="inlineStr">
         <is>
-          <t>call center</t>
+          <t>ground floor</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>8f818563-6e21-4dc5-a18b-acc8228756ce</t>
+          <t>30b72d0c-0775-40c8-81d3-18827bc0d726</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -72024,17 +72024,17 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>08:00</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>ground_floor</t>
+          <t>call_center</t>
         </is>
       </c>
       <c r="I65" t="n">
@@ -72048,14 +72048,14 @@
       </c>
       <c r="N65" t="inlineStr">
         <is>
-          <t>ground floor</t>
+          <t>call center</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>327fc4e2-ebcc-4156-a95f-58ee44c61e00</t>
+          <t>140b3ba2-e3b9-4432-9179-1c71e6c43977</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -72075,12 +72075,12 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
@@ -72106,17 +72106,17 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>bc2a4ef8-4614-4958-997f-182ca32623b3</t>
+          <t>ebfda43d-d8b9-42c3-832d-af977577f65c</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>emp_011</t>
+          <t>emp_008</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Priyanka</t>
+          <t>Anastasia</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -72126,12 +72126,12 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
           <t>16:00</t>
-        </is>
-      </c>
-      <c r="F67" t="inlineStr">
-        <is>
-          <t>20:00</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
@@ -72157,17 +72157,17 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>8b5b6c95-2ace-4e89-87cf-53cd02a64cef</t>
+          <t>68572a6c-2e2b-41e3-8218-22a8e4600643</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>emp_016</t>
+          <t>emp_008</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Arnob</t>
+          <t>Anastasia</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -72187,7 +72187,7 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>call_center</t>
+          <t>desk</t>
         </is>
       </c>
       <c r="I68" t="n">
@@ -72201,24 +72201,24 @@
       </c>
       <c r="N68" t="inlineStr">
         <is>
-          <t>call center</t>
+          <t>working from home</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>05e0548e-d8d0-4971-8080-aa4344510de6</t>
+          <t>a2bdcf06-f711-4c59-9f54-e0af06d96f5d</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>emp_016</t>
+          <t>emp_008</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Arnob</t>
+          <t>Anastasia</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -72228,12 +72228,12 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
@@ -72259,7 +72259,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>090951de-dbda-4a9d-9772-04f6e0b2ab5c</t>
+          <t>d5cdb01d-3ac6-437d-9275-ff6c2efbf381</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -72279,12 +72279,12 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>08:00</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
@@ -72310,17 +72310,17 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>f96e8944-5335-433f-a3a4-19f8ab21248a</t>
+          <t>7f4676c8-9d49-408e-8264-6739a6d9d4f3</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>emp_008</t>
+          <t>emp_016</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Anastasia</t>
+          <t>Arnob</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -72361,17 +72361,17 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>447d7fb6-281d-4188-bd11-75cf28e2d372</t>
+          <t>ca5b688f-0b40-474a-a29b-10c5108ddd67</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>emp_008</t>
+          <t>emp_016</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Anastasia</t>
+          <t>Arnob</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -72381,17 +72381,17 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>08:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>desk</t>
+          <t>call_center</t>
         </is>
       </c>
       <c r="I72" t="n">
@@ -72405,24 +72405,24 @@
       </c>
       <c r="N72" t="inlineStr">
         <is>
-          <t>working from home</t>
+          <t>call center</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>08f2274c-e59a-4299-90a3-9092fe19219f</t>
+          <t>13e78771-c8dc-43d1-a51f-2702897d5833</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>emp_008</t>
+          <t>emp_005</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Anastasia</t>
+          <t>Kavya C</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -72432,17 +72432,17 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>08:00</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>ground_floor</t>
+          <t>call_center</t>
         </is>
       </c>
       <c r="I73" t="n">
@@ -72456,14 +72456,14 @@
       </c>
       <c r="N73" t="inlineStr">
         <is>
-          <t>ground floor</t>
+          <t>call center</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>41f63817-b02d-4c3f-84b7-83a349274047</t>
+          <t>d4435f35-c3e7-4777-84b6-18dd2a47054d</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -72483,12 +72483,12 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>08:00</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
@@ -72514,7 +72514,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>4bf59dfb-a9a7-403e-80e4-a6d01fa18041</t>
+          <t>9557b90e-f154-4e70-a587-76f2cfa6be7a</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -72534,17 +72534,17 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>call_center</t>
+          <t>second_floor</t>
         </is>
       </c>
       <c r="I75" t="n">
@@ -72558,24 +72558,24 @@
       </c>
       <c r="N75" t="inlineStr">
         <is>
-          <t>call center</t>
+          <t>2nd floor</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>cc051fac-ab49-4a38-bc1e-4a81cb19d333</t>
+          <t>b0101a6b-88d9-4364-9c69-7cca6781e3d2</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>emp_005</t>
+          <t>emp_015</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Kavya C</t>
+          <t>Itohan</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -72616,7 +72616,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>953078f8-ae23-4ced-a9c2-22fa58bd3910</t>
+          <t>39243afa-bc15-4e9a-9709-9769d0a49cb3</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -72636,17 +72636,17 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>08:00</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>second_floor</t>
+          <t>call_center</t>
         </is>
       </c>
       <c r="I77" t="n">
@@ -72660,24 +72660,24 @@
       </c>
       <c r="N77" t="inlineStr">
         <is>
-          <t>2nd floor</t>
+          <t>call center</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>94d0cc82-35f9-4b08-b6ad-72b25e03b27f</t>
+          <t>457e10ff-ddaa-446b-8d46-8a716efccf6c</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>emp_015</t>
+          <t>emp_014</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Itohan</t>
+          <t>Sagar C</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -72687,17 +72687,17 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>08:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>call_center</t>
+          <t>second_floor</t>
         </is>
       </c>
       <c r="I78" t="n">
@@ -72711,24 +72711,24 @@
       </c>
       <c r="N78" t="inlineStr">
         <is>
-          <t>call center</t>
+          <t>2nd floor</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>abe425e3-207e-4504-a5d7-7693d1383450</t>
+          <t>af8dc1ac-a73a-4658-ac9b-d4cc7a3c9240</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>emp_014</t>
+          <t>emp_004</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Sagar C</t>
+          <t>Pablo</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -72738,17 +72738,17 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
           <t>16:00</t>
         </is>
       </c>
-      <c r="F79" t="inlineStr">
-        <is>
-          <t>20:00</t>
-        </is>
-      </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>second_floor</t>
+          <t>call_center</t>
         </is>
       </c>
       <c r="I79" t="n">
@@ -72762,24 +72762,24 @@
       </c>
       <c r="N79" t="inlineStr">
         <is>
-          <t>2nd floor</t>
+          <t>call center</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>841f120f-8784-48fe-af0a-d3d8b2bffa5d</t>
+          <t>43bd2a62-3ea8-4b1d-b40c-e2cffc7725f0</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>emp_004</t>
+          <t>emp_006</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Pablo</t>
+          <t>Mickaela  C</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -72820,17 +72820,17 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>02978ef1-3a3e-414f-a616-550595e898be</t>
+          <t>4616566c-4276-41d3-9563-6facf12c4100</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>emp_006</t>
+          <t>emp_003</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Mickaela  C</t>
+          <t>Nahim</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -72840,17 +72840,17 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
           <t>12:00</t>
         </is>
       </c>
-      <c r="F81" t="inlineStr">
-        <is>
-          <t>16:00</t>
-        </is>
-      </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>call_center</t>
+          <t>second_floor</t>
         </is>
       </c>
       <c r="I81" t="n">
@@ -72864,14 +72864,14 @@
       </c>
       <c r="N81" t="inlineStr">
         <is>
-          <t>call center</t>
+          <t>2nd floor</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>04f11abb-49d2-43df-8b96-3428e4ea2f4a</t>
+          <t>d387ea32-9776-4db0-8ae4-970a1e709d32</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -72891,17 +72891,17 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>08:00</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>second_floor</t>
+          <t>sixth_floor</t>
         </is>
       </c>
       <c r="I82" t="n">
@@ -72915,44 +72915,44 @@
       </c>
       <c r="N82" t="inlineStr">
         <is>
-          <t>2nd floor</t>
+          <t>6th floor</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>cb36cd9a-a055-4f08-b9e8-0770e7ad4205</t>
+          <t>d4e6179c-6c97-4026-8d33-6f483eba4cc3</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>emp_003</t>
+          <t>emp_013</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Nahim</t>
+          <t>Taran C</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>monday</t>
+          <t>tuesday</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
           <t>12:00</t>
         </is>
       </c>
-      <c r="F83" t="inlineStr">
-        <is>
-          <t>16:00</t>
-        </is>
-      </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>sixth_floor</t>
+          <t>ground_floor</t>
         </is>
       </c>
       <c r="I83" t="n">
@@ -72966,24 +72966,24 @@
       </c>
       <c r="N83" t="inlineStr">
         <is>
-          <t>6th floor</t>
+          <t>ground floor</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>5213ba0c-25d8-4760-b7dc-ede342aaaa94</t>
+          <t>6482459f-2b11-4938-9589-022911692232</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>emp_013</t>
+          <t>emp_011</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Taran C</t>
+          <t>Priyanka</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -73003,7 +73003,7 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>ground_floor</t>
+          <t>sixth_floor</t>
         </is>
       </c>
       <c r="I84" t="n">
@@ -73017,24 +73017,24 @@
       </c>
       <c r="N84" t="inlineStr">
         <is>
-          <t>ground floor</t>
+          <t>6th floor</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>f1281bc3-d585-4775-96a0-33ec17f74841</t>
+          <t>e43c9cf2-f141-43f6-9c69-86c862fdf486</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>emp_011</t>
+          <t>emp_008</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Priyanka</t>
+          <t>Anastasia</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -73054,7 +73054,7 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>sixth_floor</t>
+          <t>ground_floor</t>
         </is>
       </c>
       <c r="I85" t="n">
@@ -73068,14 +73068,14 @@
       </c>
       <c r="N85" t="inlineStr">
         <is>
-          <t>6th floor</t>
+          <t>ground floor</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>94ada7a1-6747-4f48-983d-dcb097d33a94</t>
+          <t>dd1a8de9-7935-425e-9fe0-ff3dd5b7117c</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -73126,7 +73126,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>fbe0c2ae-ae5b-4195-a47f-ed57aadf8da0</t>
+          <t>1a77c600-b7c9-4191-9ffc-f55f14ab266e</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -73177,7 +73177,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>36f163d6-0dac-4657-8cc2-ce15237f210f</t>
+          <t>f0d4e4be-c1c9-415b-bb18-f23971db2c2f</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -73228,7 +73228,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>979a4849-d0b2-4357-8aa2-badaa5207d77</t>
+          <t>58c5784e-65b3-4360-8d74-4eb7fc77e08c</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -73279,7 +73279,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>ebb17b96-475e-4463-8c27-4db711078cca</t>
+          <t>3186065a-a403-40df-9792-b040618efda3</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -73330,7 +73330,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>5498b6d6-c6fa-48c7-80bf-9d72c9732044</t>
+          <t>b360b1ef-666d-47d4-acaa-8d3dfc872073</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -73381,7 +73381,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>f98ba93f-24da-4a2b-b0be-421bb9cd9bcc</t>
+          <t>dd4ee70b-1302-4298-8846-8524c668366d</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -73432,7 +73432,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>7ba368cb-b423-4542-8046-aa7539683667</t>
+          <t>06c541bc-e571-42b2-8f7f-4c654597b267</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -73483,7 +73483,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>7549f6cc-dcbf-4501-b416-c5c68702a97c</t>
+          <t>eb79295d-454d-4cb4-8e7f-e2e6bf3dbaa5</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -73534,7 +73534,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>ad62566c-72c2-49bf-b6d3-d3f2d8b166de</t>
+          <t>afcb1dfa-6e03-414b-a109-f6f48afe31d8</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -73585,7 +73585,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>5498c591-efd7-446d-b832-affd3cf48369</t>
+          <t>4b80de8f-bf26-48ad-a319-81b6b1d2b259</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -73636,7 +73636,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>1b5f8957-39a3-49c3-ba03-27197d3389a9</t>
+          <t>adcf72ab-4add-49a7-9298-cabb4c3d1fd6</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -73687,7 +73687,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>2d01ccd4-8743-4f26-9a35-04fa21b4827f</t>
+          <t>e93befa7-909e-4076-a838-124a21a088a0</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -73738,7 +73738,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>b48bb0db-2c9d-4838-a2c6-ec65bc877109</t>
+          <t>95218e12-9ea4-43ae-894a-4d7b1adc3a31</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -73789,7 +73789,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>42cf3024-95f9-46fd-b244-290f7720aa6a</t>
+          <t>e60d0fac-8bb5-4bf8-9e48-9562c1cab55e</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -73840,7 +73840,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>339e34b9-8ab7-40cf-935a-9e523acea460</t>
+          <t>6926e0bb-df80-4380-b10b-bfba3e8cf685</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -73891,7 +73891,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>e5caf1e4-b9c6-4d72-9d51-f5af5bd4d573</t>
+          <t>00a5a979-c044-44c8-8af0-0fe977df48e6</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -73936,164 +73936,6 @@
       <c r="N102" t="inlineStr">
         <is>
           <t>manager activities</t>
-        </is>
-      </c>
-    </row>
-    <row r="103">
-      <c r="A103" t="inlineStr">
-        <is>
-          <t>locked_d4aaa49b-72e3-4e1c-9db0-c68ab1ca966f_2026-06-22</t>
-        </is>
-      </c>
-      <c r="B103" t="inlineStr">
-        <is>
-          <t>emp_1781047684821</t>
-        </is>
-      </c>
-      <c r="C103" t="inlineStr">
-        <is>
-          <t>Test New Worker</t>
-        </is>
-      </c>
-      <c r="D103" t="inlineStr">
-        <is>
-          <t>monday</t>
-        </is>
-      </c>
-      <c r="E103" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="F103" t="inlineStr">
-        <is>
-          <t>23:59</t>
-        </is>
-      </c>
-      <c r="G103" t="inlineStr">
-        <is>
-          <t>desk</t>
-        </is>
-      </c>
-      <c r="I103" t="n">
-        <v>23.98333333333333</v>
-      </c>
-      <c r="J103" t="b">
-        <v>0</v>
-      </c>
-      <c r="L103" t="b">
-        <v>1</v>
-      </c>
-      <c r="M103" t="inlineStr">
-        <is>
-          <t>Day Off</t>
-        </is>
-      </c>
-      <c r="N103" t="inlineStr">
-        <is>
-          <t>day off</t>
-        </is>
-      </c>
-    </row>
-    <row r="104">
-      <c r="A104" t="inlineStr">
-        <is>
-          <t>locked_365e0a5b-8b06-4ca7-a1c8-92c4eb3bd061_2026-06-23</t>
-        </is>
-      </c>
-      <c r="B104" t="inlineStr">
-        <is>
-          <t>emp_1781047684821</t>
-        </is>
-      </c>
-      <c r="C104" t="inlineStr">
-        <is>
-          <t>Test New Worker</t>
-        </is>
-      </c>
-      <c r="D104" t="inlineStr">
-        <is>
-          <t>tuesday</t>
-        </is>
-      </c>
-      <c r="E104" t="inlineStr">
-        <is>
-          <t>09:00</t>
-        </is>
-      </c>
-      <c r="F104" t="inlineStr">
-        <is>
-          <t>12:00</t>
-        </is>
-      </c>
-      <c r="G104" t="inlineStr">
-        <is>
-          <t>desk</t>
-        </is>
-      </c>
-      <c r="I104" t="n">
-        <v>3</v>
-      </c>
-      <c r="J104" t="b">
-        <v>0</v>
-      </c>
-      <c r="L104" t="b">
-        <v>1</v>
-      </c>
-      <c r="M104" t="inlineStr">
-        <is>
-          <t>09:00 - 12:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="105">
-      <c r="A105" t="inlineStr">
-        <is>
-          <t>locked_db51084f-522f-4856-9371-22fcafe50cbf_2026-06-24</t>
-        </is>
-      </c>
-      <c r="B105" t="inlineStr">
-        <is>
-          <t>emp_1781047684821</t>
-        </is>
-      </c>
-      <c r="C105" t="inlineStr">
-        <is>
-          <t>Test New Worker</t>
-        </is>
-      </c>
-      <c r="D105" t="inlineStr">
-        <is>
-          <t>wednesday</t>
-        </is>
-      </c>
-      <c r="E105" t="inlineStr">
-        <is>
-          <t>09:00</t>
-        </is>
-      </c>
-      <c r="F105" t="inlineStr">
-        <is>
-          <t>15:00</t>
-        </is>
-      </c>
-      <c r="G105" t="inlineStr">
-        <is>
-          <t>desk</t>
-        </is>
-      </c>
-      <c r="I105" t="n">
-        <v>6</v>
-      </c>
-      <c r="J105" t="b">
-        <v>0</v>
-      </c>
-      <c r="L105" t="b">
-        <v>1</v>
-      </c>
-      <c r="M105" t="inlineStr">
-        <is>
-          <t>09:00 - 15:00</t>
         </is>
       </c>
     </row>
@@ -74109,7 +73951,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N97"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -78858,7 +78700,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:AA36"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="35.5" customWidth="1" min="2" max="2"/>
@@ -80404,7 +80246,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:V35"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -81906,7 +81748,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:V36"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -83308,7 +83150,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:V33"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>

</xml_diff>

<commit_message>
Block auto-generate without events and add debug logging for time restrictions
</commit_message>
<xml_diff>
--- a/api/backend/uploads/ibu_schedule.xlsx
+++ b/api/backend/uploads/ibu_schedule.xlsx
@@ -3148,7 +3148,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:V39"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -4756,7 +4756,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:V34"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -6255,7 +6255,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:V34"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -7697,7 +7697,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:V33"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -9043,7 +9043,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:V33"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -10485,7 +10485,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:V33"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -11953,7 +11953,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:V33"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -13287,7 +13287,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:U32"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="18.1640625" customWidth="1" min="2" max="2"/>
@@ -14646,7 +14646,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:U32"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -16008,7 +16008,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:U32"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -17354,7 +17354,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:U32"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -18724,7 +18724,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:V39"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -20307,7 +20307,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:U31"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -21597,7 +21597,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:U31"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -22938,7 +22938,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:U33"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="19.5" customWidth="1" min="2" max="2"/>
@@ -24398,7 +24398,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:U33"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -25731,7 +25731,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:U32"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -27006,7 +27006,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:Q31"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -28201,7 +28201,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:Q33"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -29503,7 +29503,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:Q33"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -30826,7 +30826,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:Q33"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -32127,7 +32127,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:Q33"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -33362,7 +33362,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:V39"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
@@ -34919,7 +34919,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:Q34"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -36183,7 +36183,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:Q34"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -37440,7 +37440,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:Q31"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -38517,7 +38517,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:Q31"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -39571,7 +39571,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:Q23"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -40623,7 +40623,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:Q24"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -41673,7 +41673,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:R24"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -42746,7 +42746,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:Q24"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -43797,7 +43797,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:Q23"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -44827,7 +44827,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:Q21"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -45769,7 +45769,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:V39"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -47276,7 +47276,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:P22"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -48259,7 +48259,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:Q21"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="17.5" customWidth="1" min="1" max="2"/>
     <col width="4.33203125" customWidth="1" min="3" max="3"/>
@@ -49176,7 +49176,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:Q23"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -50278,7 +50278,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:Q24"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="11.1640625" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -52154,7 +52154,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N97"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -67189,7 +67189,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:V36"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -68698,7 +68698,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N102"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -68791,7 +68791,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ddf6b6c6-8759-4a7f-8b74-c04db71a445d</t>
+          <t>6b248f7e-5284-46a0-91f5-2daa33cd5455</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -68842,7 +68842,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>c53aec0d-5261-44cb-8063-8b78aa585c65</t>
+          <t>cd988095-4bea-4a1f-b759-108212c75fbb</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -68893,7 +68893,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>cbfc45a5-2262-43ac-a81d-aac7536af2f0</t>
+          <t>3ac5ed3a-eeb2-45eb-b3ef-dddd504f46a4</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -68944,7 +68944,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>8d04c852-7d73-4204-ab7f-177774eefcac</t>
+          <t>5ffcdbce-d203-4659-8fbd-47d410db228f</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -68995,7 +68995,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>9de14841-c639-4b19-b00a-66a5dac4deb3</t>
+          <t>b098cdf7-37b1-4af9-9176-344cb06b0d9e</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -69046,7 +69046,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>8357d5f9-b465-4b9f-bbc4-79bc9bc7a5ed</t>
+          <t>c262366f-1e92-41c6-a67b-df1a7611848c</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -69097,7 +69097,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>428a3d17-8f63-4aea-b1ad-99b3c8f69afd</t>
+          <t>0b93bbc9-993b-4588-af0e-d8747f428638</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -69148,7 +69148,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>19a431be-cd64-4460-ba71-b783c1ab010d</t>
+          <t>ae596dcb-409f-4640-a33d-12dbb0ffeae9</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -69199,7 +69199,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>bd83aa05-e768-4d79-a664-74726d0e3dd0</t>
+          <t>c1f68198-8e6c-46dd-8b24-5ad57b914e0c</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -69250,7 +69250,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>d77bfe77-dfa0-4ce4-8b2c-4992807224ad</t>
+          <t>257d8630-9abe-41bc-bf0a-61fddcae0e7d</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -69301,7 +69301,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>c42d9d26-3276-4072-9cc6-23eb03a98da0</t>
+          <t>55a3a90e-a777-4919-af57-a14f5dc66edd</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -69352,7 +69352,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>31c11537-631f-4949-b110-56f5ffcba1dc</t>
+          <t>7c39a769-b42f-447c-9a84-4abbb1ae76be</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -69403,7 +69403,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>f560f98f-7bb7-4fef-a0b9-fb27941cc934</t>
+          <t>fd991ff0-f073-4b98-8535-73174a32963b</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -69454,7 +69454,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>82d4ce62-f524-47d4-9f69-779b6b6aa6fe</t>
+          <t>4b3efafa-06da-41c0-9a3b-83b43ed4d937</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -69505,7 +69505,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>a8a87db0-eee2-4453-aac6-25014a442431</t>
+          <t>a96d7d28-0993-4778-a16e-ac6ee2e7def5</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -69556,7 +69556,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>5bb297f8-5e30-47c0-8b2e-29bdd6a01fbb</t>
+          <t>cc0a30f3-a59f-49d3-9ba0-27c4da12213a</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -69607,7 +69607,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>87396322-661a-45dd-ad4e-b9f7b8371e0c</t>
+          <t>bd825e9a-d542-4a0e-9e70-1105481b7329</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -69658,7 +69658,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>7b45cf91-2cf0-4621-b000-78b4d2e37129</t>
+          <t>aa879098-ba45-49bf-81dc-a3b2b4edfcc6</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -69709,7 +69709,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>655ad4b3-b52c-40cf-b4ef-d3f7ee419944</t>
+          <t>f6dbc4ab-5caa-4ecd-90c8-6dc02307a627</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -69760,7 +69760,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>521f28b6-100f-48b3-8614-b0c185d95ff7</t>
+          <t>dfab11f1-6e65-45fd-a8e7-c62b0091416a</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -69811,7 +69811,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>bd52963d-a32b-4975-9362-3c391716b35b</t>
+          <t>66310678-aba2-451b-ba24-594421e154b1</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -69862,7 +69862,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>f40fec7f-b9bc-4d20-9267-fda12c7c17aa</t>
+          <t>e2cca692-7e8d-4e03-a25a-28498fecc08d</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -69913,7 +69913,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>fef8cf86-6271-42c4-b4bc-46e0ad1f7fa9</t>
+          <t>1d66699b-2d14-46d6-aec8-5b2db11d2d11</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -69964,7 +69964,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>9fc903d4-bc15-4ca2-a421-e7034794ef60</t>
+          <t>168c3127-7a70-4895-80f4-dc21d3152076</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -70015,7 +70015,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>93f9ce83-50bc-4a48-ba7e-deccd721e240</t>
+          <t>6b20a4e6-ac19-41d6-a7d8-f9a80b312ba4</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -70066,7 +70066,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>9239e818-4083-4d34-93d6-2b78dea8592c</t>
+          <t>20e4ed2b-801f-4f99-b4f9-1bbaccf123c7</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -70117,7 +70117,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>04c52363-1a46-4168-9337-7714659e1199</t>
+          <t>c6888d3e-2b73-46ee-bf32-c391a4371e53</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -70168,7 +70168,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>1ab12f6c-3d25-4bd7-982b-340de0cd8b20</t>
+          <t>c4f16c47-0621-4808-8291-c5df2b8b9c99</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -70219,7 +70219,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>1eb53ccb-eeeb-48ed-8c88-e277bdf795b3</t>
+          <t>912e7fd2-62a4-4dec-a0c7-26946b4106ad</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -70270,7 +70270,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2290f47f-fa94-4397-88b5-908959f44c87</t>
+          <t>7e44a40c-f98d-4fd3-8d99-1093118d92d4</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -70321,7 +70321,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>3ce1b20b-d65d-4c5b-a7c8-f9db5357f19b</t>
+          <t>5c1250a6-9804-464a-885d-b28b81cc08ae</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -70372,7 +70372,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>57510fef-b553-428a-b2ab-c528d2c4a175</t>
+          <t>9e359256-f7a4-4ad1-a666-2c37afb0eed4</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -70423,7 +70423,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>a5dea3db-bfed-422a-8432-909dcb259fcc</t>
+          <t>f7c69a86-0f39-4cd0-82b4-f88153391ef1</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -70474,7 +70474,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>e979c654-b81a-414c-8e55-cb1cbf31a196</t>
+          <t>a00450aa-64a0-41d3-ad68-2f2d3a855ebe</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -70525,7 +70525,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>413fec59-af83-4d29-bf95-816b2cfcffff</t>
+          <t>e4ca2275-1c31-45f9-97d9-ed3792a4c42f</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -70576,7 +70576,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>07021605-7a1b-45d4-8794-d592ab95c3c5</t>
+          <t>01787626-12f7-4cf1-8ac9-e3fc7a9ef856</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -70627,7 +70627,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>4f64639c-5421-418f-8bb1-157db36d2b06</t>
+          <t>3bcfb7b8-fdc9-43bb-b69e-32a55079bc54</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -70678,7 +70678,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>bd428c34-fbd0-489f-8d61-151a1023b2f7</t>
+          <t>234ee56b-8907-434a-846c-7b5a12b6c163</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -70729,7 +70729,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>a5cc59dc-f7a7-4f67-a6df-a1a8639eb69b</t>
+          <t>11877578-a900-4bc9-8327-337e6fd75051</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -70780,7 +70780,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>fb498cd6-c381-4013-844e-8d7e14f6fcf3</t>
+          <t>28bd713a-42c7-483d-af76-51c4c60bb87e</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -70831,7 +70831,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>4f28a7be-cd9f-407e-b0ae-da819eb6a2f1</t>
+          <t>fcc5fab1-5650-4643-b0e9-6feaf453e3a4</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -70882,7 +70882,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>20f08772-6031-49ab-9b47-b13cd7f88ced</t>
+          <t>e4818ada-f9bf-4d88-b698-e2eed89c7a31</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -70933,7 +70933,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>e14f3ac8-8bb9-4f89-a75d-cbc4ea395d0f</t>
+          <t>678ec2d0-69da-4eb9-a277-ebff39e0fc93</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -70984,7 +70984,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>24eb5a97-ea2a-4f9b-b7ac-208c20f578ae</t>
+          <t>28650c26-ebbc-467c-91d3-9e478792c4c9</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -71035,7 +71035,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>54279a42-4f83-4eed-b383-6c0f834141ee</t>
+          <t>9e0456c7-e0e7-4ebf-bac1-d8b59c492b88</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -71086,7 +71086,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>28bf11cd-57ea-40a4-a4f9-86b8d958b763</t>
+          <t>6261579f-97d9-435f-ad4e-ae63d98adff9</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -71137,7 +71137,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>b32be596-e7f5-4c73-b7a0-6cb27165d849</t>
+          <t>87a90e5e-5630-42c5-bff5-4b3c1df71f62</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -71188,7 +71188,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>bf3a77c1-494d-4903-b11c-3ee6f237ac64</t>
+          <t>f73e15f0-4f29-47b4-8e92-5dd92adc80e7</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -71239,7 +71239,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>19d74442-de67-47ec-8353-41f01f480ea1</t>
+          <t>c3ff8acd-d83c-4fee-b531-baaf4b228c7a</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -71290,7 +71290,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>246f0e9a-d44f-43a2-acc7-02fbd0081dcf</t>
+          <t>98510673-6d24-4846-9566-49dd2a01d02c</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -71341,7 +71341,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>724ed3f8-698a-4cb8-8f2d-b1b3307559eb</t>
+          <t>417c77c2-eadd-4622-acca-33258ef41f6e</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -71392,7 +71392,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>c723f8c4-beaf-46b7-9b8c-af4704e6c4f4</t>
+          <t>03ad8020-c2ce-4eb3-8f5a-61386a101f4a</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -71443,7 +71443,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>ccca2b37-242a-4f98-b404-a656a5b366df</t>
+          <t>e566f726-1ce3-4723-a671-349875cb0e49</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -71494,7 +71494,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>03e5df37-d433-4e7c-8b80-a58440f3f300</t>
+          <t>c44a26c6-7ac2-47b3-8729-da6ef13b01ac</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -71545,7 +71545,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>e2520c08-ff5e-4f43-b847-68e744f3afda</t>
+          <t>a1a4ffbd-c655-4323-b822-01255b59838d</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -71596,7 +71596,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>b5663478-c85a-4e73-b0b2-c84e00d4d1bb</t>
+          <t>4bd0d53d-77db-4f85-a8a0-1d81a2e2b949</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -71647,7 +71647,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>d66bf4ab-5075-4d36-852a-341a583d3e3f</t>
+          <t>8488ccf0-20eb-436e-84ef-b5f12179e498</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -71698,7 +71698,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>e688220d-3a04-4062-8f41-7e84f1f25fa8</t>
+          <t>0eeb4d7b-583e-436a-8758-454a071e55bf</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -71749,7 +71749,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>862a3073-d1f5-419e-9ac2-f6f2e5b6fd60</t>
+          <t>abd0e436-199b-4e3c-a7a0-b27bbade7781</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -71800,7 +71800,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>60055902-d777-47bf-9533-3f5b1fbaaa94</t>
+          <t>8f8942af-c930-4100-881a-e96a4f95983f</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -71851,7 +71851,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>dd291705-2dfb-438c-a2fe-a48d1ace8664</t>
+          <t>ff2ed429-0202-404e-8b5f-324e14bb4b6a</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -71902,7 +71902,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>ca31c341-2358-4210-ba23-3d2cb3c2e4a0</t>
+          <t>5cdd23ff-5089-45fc-b9cb-e1110a649f75</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -71953,7 +71953,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>21b5c4d1-46db-4119-a8ab-476365be56be</t>
+          <t>534dd986-2da6-4dd4-a2ec-3f19cd7fbec1</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -72004,7 +72004,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>30b72d0c-0775-40c8-81d3-18827bc0d726</t>
+          <t>31d1dc70-4d42-4c2f-b3e8-1d0c3053ec5d</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -72055,7 +72055,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>140b3ba2-e3b9-4432-9179-1c71e6c43977</t>
+          <t>17b8aba4-52e3-455d-8c2d-0d62216096fe</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -72106,7 +72106,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>ebfda43d-d8b9-42c3-832d-af977577f65c</t>
+          <t>1dc9389c-f4e6-4fb6-ba2b-6369a6382b54</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -72157,7 +72157,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>68572a6c-2e2b-41e3-8218-22a8e4600643</t>
+          <t>8d673311-c98b-444e-878a-814a55087583</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -72208,7 +72208,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>a2bdcf06-f711-4c59-9f54-e0af06d96f5d</t>
+          <t>ec0c0a25-2459-4227-bb0e-6aa2951d289b</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -72259,7 +72259,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>d5cdb01d-3ac6-437d-9275-ff6c2efbf381</t>
+          <t>abf428eb-e881-426d-a6ab-fa5a9d224df2</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -72310,7 +72310,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>7f4676c8-9d49-408e-8264-6739a6d9d4f3</t>
+          <t>d57494c7-6350-4547-9b32-6e692b8c8e91</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -72361,7 +72361,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>ca5b688f-0b40-474a-a29b-10c5108ddd67</t>
+          <t>49159b7c-f1ee-484b-bdfa-5a37856d6e3f</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -72412,7 +72412,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>13e78771-c8dc-43d1-a51f-2702897d5833</t>
+          <t>ca434ee8-638f-41e1-b9d2-73a11cd4ce87</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -72463,7 +72463,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>d4435f35-c3e7-4777-84b6-18dd2a47054d</t>
+          <t>c65e177a-671b-49e2-8108-8601ffbae1a3</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -72514,7 +72514,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>9557b90e-f154-4e70-a587-76f2cfa6be7a</t>
+          <t>fcc5933e-49e6-4d59-930b-b94d8c7bd833</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -72565,7 +72565,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>b0101a6b-88d9-4364-9c69-7cca6781e3d2</t>
+          <t>da2f8964-fd47-4987-b5c7-d1d87ed823e0</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -72616,7 +72616,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>39243afa-bc15-4e9a-9709-9769d0a49cb3</t>
+          <t>04c10bf3-7854-4f85-b0aa-eadb0c4014b6</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -72667,7 +72667,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>457e10ff-ddaa-446b-8d46-8a716efccf6c</t>
+          <t>dfa113d5-cf0c-45d7-ab77-8a1664130a63</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -72718,7 +72718,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>af8dc1ac-a73a-4658-ac9b-d4cc7a3c9240</t>
+          <t>e2bc50ae-b88c-4503-aa4f-c5d2882b93ad</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -72769,7 +72769,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>43bd2a62-3ea8-4b1d-b40c-e2cffc7725f0</t>
+          <t>f7409aa9-8811-4292-ab1c-d8552a331482</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -72820,7 +72820,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>4616566c-4276-41d3-9563-6facf12c4100</t>
+          <t>3bf0de50-336f-4e9b-be0f-0a874f90bc8e</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -72871,7 +72871,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>d387ea32-9776-4db0-8ae4-970a1e709d32</t>
+          <t>c3cba96f-6dbf-4d64-97ef-2ed1685445c0</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -72922,7 +72922,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>d4e6179c-6c97-4026-8d33-6f483eba4cc3</t>
+          <t>2a355782-2cca-4ea6-909d-8e810eb7cea8</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -72973,7 +72973,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>6482459f-2b11-4938-9589-022911692232</t>
+          <t>851215f4-6436-4332-9e32-693366e1c33d</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -73024,7 +73024,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>e43c9cf2-f141-43f6-9c69-86c862fdf486</t>
+          <t>b83a40c4-ba8e-4010-8509-7c607834a571</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -73075,7 +73075,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>dd1a8de9-7935-425e-9fe0-ff3dd5b7117c</t>
+          <t>cc2dd004-f746-4ebc-8b05-3ec8fb1537c0</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -73126,7 +73126,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>1a77c600-b7c9-4191-9ffc-f55f14ab266e</t>
+          <t>f763d3ef-d90e-44fc-937a-3f4a24a1fb6f</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -73177,7 +73177,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>f0d4e4be-c1c9-415b-bb18-f23971db2c2f</t>
+          <t>f414166f-969f-45d7-9ac2-610218a03613</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -73228,7 +73228,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>58c5784e-65b3-4360-8d74-4eb7fc77e08c</t>
+          <t>d7f5d3fc-cdb8-4fba-9f7f-72fb98a62977</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -73279,7 +73279,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>3186065a-a403-40df-9792-b040618efda3</t>
+          <t>f4502a34-aafa-459b-9db9-1262087907ec</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -73330,7 +73330,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>b360b1ef-666d-47d4-acaa-8d3dfc872073</t>
+          <t>1c4ddc5d-9224-4d46-b20e-0f547d5b2175</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -73381,7 +73381,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>dd4ee70b-1302-4298-8846-8524c668366d</t>
+          <t>927479fa-1228-4a71-ad77-1a68603e8978</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -73432,7 +73432,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>06c541bc-e571-42b2-8f7f-4c654597b267</t>
+          <t>6456d93a-a2c7-4632-a056-d06d25715770</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -73483,7 +73483,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>eb79295d-454d-4cb4-8e7f-e2e6bf3dbaa5</t>
+          <t>cf2b59c3-0f33-4253-a7c2-758139738869</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -73534,7 +73534,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>afcb1dfa-6e03-414b-a109-f6f48afe31d8</t>
+          <t>f35e1c17-4711-442f-bdc1-6efc21e03dae</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -73585,7 +73585,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>4b80de8f-bf26-48ad-a319-81b6b1d2b259</t>
+          <t>937ef8a7-4cf0-4db3-ba71-0c7e1a0ce944</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -73636,7 +73636,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>adcf72ab-4add-49a7-9298-cabb4c3d1fd6</t>
+          <t>d451aad2-8a10-4a2e-8277-a201b0488c90</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -73687,7 +73687,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>e93befa7-909e-4076-a838-124a21a088a0</t>
+          <t>333fcb62-c2a2-4478-98ef-467291a14323</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -73738,7 +73738,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>95218e12-9ea4-43ae-894a-4d7b1adc3a31</t>
+          <t>bc7f97aa-0a10-40ea-8b04-98269ba5173c</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -73789,7 +73789,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>e60d0fac-8bb5-4bf8-9e48-9562c1cab55e</t>
+          <t>0a23e5d2-8960-4b31-b504-14dc9190e5e8</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -73840,7 +73840,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>6926e0bb-df80-4380-b10b-bfba3e8cf685</t>
+          <t>e349aafa-cf8b-47c3-9093-38435e0b5a44</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -73891,7 +73891,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>00a5a979-c044-44c8-8af0-0fe977df48e6</t>
+          <t>90d19402-295a-4d3c-8c4f-f5bed5e03dba</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -73951,7 +73951,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N97"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -78700,7 +78700,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:AA36"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="35.5" customWidth="1" min="2" max="2"/>
@@ -80246,7 +80246,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:V35"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -81748,7 +81748,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:V36"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>
@@ -83150,7 +83150,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:V33"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26.5" customWidth="1" min="1" max="1"/>
     <col width="17.5" customWidth="1" min="2" max="2"/>

</xml_diff>

<commit_message>
Add employee preferences tab for managers with priority over employee preferences
</commit_message>
<xml_diff>
--- a/api/backend/uploads/ibu_schedule.xlsx
+++ b/api/backend/uploads/ibu_schedule.xlsx
@@ -57156,7 +57156,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -57317,6 +57317,50 @@
       </c>
       <c r="K3" s="463" t="n">
         <v>46182.68622203704</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>event_03da33df</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Party</t>
+        </is>
+      </c>
+      <c r="C4" s="462" t="n">
+        <v>46195</v>
+      </c>
+      <c r="D4" s="462" t="n">
+        <v>46183</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>22:00</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>ground floor</t>
+        </is>
+      </c>
+      <c r="H4" t="n">
+        <v>2</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>emp_1780946033840</t>
+        </is>
+      </c>
+      <c r="K4" s="463" t="n">
+        <v>46183.38671530093</v>
       </c>
     </row>
   </sheetData>
@@ -68791,7 +68835,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>6b248f7e-5284-46a0-91f5-2daa33cd5455</t>
+          <t>7ff7b0d2-6351-44e2-bf85-510fc959688e</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -68842,7 +68886,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>cd988095-4bea-4a1f-b759-108212c75fbb</t>
+          <t>45df558a-aa69-4dd6-b4e1-022c0a972b6d</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -68893,7 +68937,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>3ac5ed3a-eeb2-45eb-b3ef-dddd504f46a4</t>
+          <t>d42791c1-6ca9-4bdb-aad2-13ae5d06e092</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -68944,7 +68988,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>5ffcdbce-d203-4659-8fbd-47d410db228f</t>
+          <t>13588e7d-f57f-4525-8982-e773f0ed97c1</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -68995,7 +69039,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>b098cdf7-37b1-4af9-9176-344cb06b0d9e</t>
+          <t>1e218a84-a42a-43b5-b3fc-d917fad44617</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -69046,7 +69090,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>c262366f-1e92-41c6-a67b-df1a7611848c</t>
+          <t>53e8c907-2fd3-44a9-bd5a-4fd84d09723d</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -69097,7 +69141,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0b93bbc9-993b-4588-af0e-d8747f428638</t>
+          <t>2352b86b-7401-4640-9f06-65c823953b7f</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -69148,7 +69192,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ae596dcb-409f-4640-a33d-12dbb0ffeae9</t>
+          <t>2d96ea5d-27fe-4f35-a73f-f77962cedcdf</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -69199,7 +69243,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>c1f68198-8e6c-46dd-8b24-5ad57b914e0c</t>
+          <t>842785ca-04e7-4d0f-b2dd-b9f1c40c7f3d</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -69250,7 +69294,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>257d8630-9abe-41bc-bf0a-61fddcae0e7d</t>
+          <t>34721286-124f-497a-a46e-1feffb14eac9</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -69301,7 +69345,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>55a3a90e-a777-4919-af57-a14f5dc66edd</t>
+          <t>7ad451ea-f4a6-4063-b115-747b543475d6</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -69352,7 +69396,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>7c39a769-b42f-447c-9a84-4abbb1ae76be</t>
+          <t>0d1b374c-063a-43e5-b21e-400dd9c5c168</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -69403,7 +69447,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>fd991ff0-f073-4b98-8535-73174a32963b</t>
+          <t>3eba25aa-98f0-47db-9efb-3b164e5ae301</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -69454,7 +69498,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>4b3efafa-06da-41c0-9a3b-83b43ed4d937</t>
+          <t>f8b27537-1913-4060-857d-3379c6d7f4b3</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -69505,7 +69549,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>a96d7d28-0993-4778-a16e-ac6ee2e7def5</t>
+          <t>c844bef3-e2ce-473a-8e11-fef1b4643dac</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -69556,7 +69600,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>cc0a30f3-a59f-49d3-9ba0-27c4da12213a</t>
+          <t>600762e7-7982-40be-b3d9-01dbb4a76dad</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -69607,7 +69651,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>bd825e9a-d542-4a0e-9e70-1105481b7329</t>
+          <t>93df729a-4f9a-45e6-89db-4856679b2b96</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -69658,7 +69702,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>aa879098-ba45-49bf-81dc-a3b2b4edfcc6</t>
+          <t>dfbe2b4e-dac8-4d1f-9d86-a9874b9f6856</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -69709,7 +69753,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>f6dbc4ab-5caa-4ecd-90c8-6dc02307a627</t>
+          <t>57fc8acb-d648-4b6a-9197-6db671656ca0</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -69760,7 +69804,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>dfab11f1-6e65-45fd-a8e7-c62b0091416a</t>
+          <t>df36ea6f-1637-4c2d-ad13-226eb5d07444</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -69811,7 +69855,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>66310678-aba2-451b-ba24-594421e154b1</t>
+          <t>cde1197a-ce15-40b2-ac78-bcb34f7f188a</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -69862,7 +69906,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>e2cca692-7e8d-4e03-a25a-28498fecc08d</t>
+          <t>72e14c1b-bf88-40a2-be94-5ffb90a35ad7</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -69913,7 +69957,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>1d66699b-2d14-46d6-aec8-5b2db11d2d11</t>
+          <t>0e681346-8112-442d-ae07-1447a4bfa50a</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -69964,7 +70008,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>168c3127-7a70-4895-80f4-dc21d3152076</t>
+          <t>99195d2f-6e30-49a6-bcd3-581b8ac08e27</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -70015,7 +70059,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>6b20a4e6-ac19-41d6-a7d8-f9a80b312ba4</t>
+          <t>f522649b-cb81-4066-96f5-091219ccb865</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -70066,7 +70110,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>20e4ed2b-801f-4f99-b4f9-1bbaccf123c7</t>
+          <t>2d2730d7-3d4c-4998-a055-93403b9a0bf0</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -70117,7 +70161,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>c6888d3e-2b73-46ee-bf32-c391a4371e53</t>
+          <t>650651bc-97b5-4ec2-96da-6855f4b5aafc</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -70168,7 +70212,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>c4f16c47-0621-4808-8291-c5df2b8b9c99</t>
+          <t>75f66d6f-6619-496c-8a74-d58146e3dce6</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -70219,7 +70263,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>912e7fd2-62a4-4dec-a0c7-26946b4106ad</t>
+          <t>0ac796e4-751e-4b84-94b2-c125ad110c6c</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -70270,7 +70314,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>7e44a40c-f98d-4fd3-8d99-1093118d92d4</t>
+          <t>f113a1da-d3fb-4c90-88f1-4899753f00e3</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -70321,7 +70365,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>5c1250a6-9804-464a-885d-b28b81cc08ae</t>
+          <t>30b9c114-6052-4213-8f71-71266d2b69f7</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -70372,7 +70416,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>9e359256-f7a4-4ad1-a666-2c37afb0eed4</t>
+          <t>71d01d5d-32ac-4928-8be9-331c6356a329</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -70423,7 +70467,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>f7c69a86-0f39-4cd0-82b4-f88153391ef1</t>
+          <t>cbfed06b-55cb-44ca-b2f4-ab07974c0dc2</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -70474,7 +70518,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>a00450aa-64a0-41d3-ad68-2f2d3a855ebe</t>
+          <t>169719f1-6c0c-4d1d-8213-3798f66b77e6</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -70525,7 +70569,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>e4ca2275-1c31-45f9-97d9-ed3792a4c42f</t>
+          <t>7e2ced87-9f25-4d3e-9d23-414c859853f7</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -70576,7 +70620,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>01787626-12f7-4cf1-8ac9-e3fc7a9ef856</t>
+          <t>4d93f403-f186-4e24-b83e-3789dcfedd29</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -70627,7 +70671,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>3bcfb7b8-fdc9-43bb-b69e-32a55079bc54</t>
+          <t>decb71ba-dbf8-4e5d-a07c-27a8480c7c97</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -70678,7 +70722,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>234ee56b-8907-434a-846c-7b5a12b6c163</t>
+          <t>5b35b462-4309-4edc-af41-07ba25722cfa</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -70729,7 +70773,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>11877578-a900-4bc9-8327-337e6fd75051</t>
+          <t>7496d006-2c40-4329-acfd-28b9d5419f95</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -70780,7 +70824,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>28bd713a-42c7-483d-af76-51c4c60bb87e</t>
+          <t>85e76bef-1958-4df8-8210-bb94e441be38</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -70831,7 +70875,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>fcc5fab1-5650-4643-b0e9-6feaf453e3a4</t>
+          <t>cc49d32b-1ba9-49d6-a2a8-c375875c1bdc</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -70882,7 +70926,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>e4818ada-f9bf-4d88-b698-e2eed89c7a31</t>
+          <t>41fbffa1-4361-4df3-96f2-53b58adce91b</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -70933,7 +70977,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>678ec2d0-69da-4eb9-a277-ebff39e0fc93</t>
+          <t>069e937c-cf33-4a8f-87e6-c724fd97e033</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -70984,7 +71028,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>28650c26-ebbc-467c-91d3-9e478792c4c9</t>
+          <t>33af01f0-1048-428f-858a-cfceda38832e</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -71035,7 +71079,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>9e0456c7-e0e7-4ebf-bac1-d8b59c492b88</t>
+          <t>6819214d-7115-4f49-a122-fc59c1f8b170</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -71086,7 +71130,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>6261579f-97d9-435f-ad4e-ae63d98adff9</t>
+          <t>25fccba8-049e-458a-b07a-3f5133e1ea97</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -71137,7 +71181,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>87a90e5e-5630-42c5-bff5-4b3c1df71f62</t>
+          <t>180ab3c3-9c43-423a-ac81-a1a949682cbb</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -71188,7 +71232,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>f73e15f0-4f29-47b4-8e92-5dd92adc80e7</t>
+          <t>e455f7ba-af99-4e09-9971-a48335e331ce</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -71239,7 +71283,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>c3ff8acd-d83c-4fee-b531-baaf4b228c7a</t>
+          <t>68f064b8-6077-4c3b-807f-99543119eb15</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -71290,7 +71334,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>98510673-6d24-4846-9566-49dd2a01d02c</t>
+          <t>43b82a7b-b625-4eda-9cd5-fc38c728d018</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -71341,7 +71385,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>417c77c2-eadd-4622-acca-33258ef41f6e</t>
+          <t>b25653b0-91d5-4dcb-9932-5b72d232fb65</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -71392,7 +71436,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>03ad8020-c2ce-4eb3-8f5a-61386a101f4a</t>
+          <t>bf291c3f-c5cf-4066-85a1-f6924d8881f1</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -71443,7 +71487,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>e566f726-1ce3-4723-a671-349875cb0e49</t>
+          <t>c8469c1c-f6e7-4044-968b-a64e308246a2</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -71494,7 +71538,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>c44a26c6-7ac2-47b3-8729-da6ef13b01ac</t>
+          <t>da5b1700-50e3-4f1c-a431-0624482f8378</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -71545,7 +71589,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>a1a4ffbd-c655-4323-b822-01255b59838d</t>
+          <t>0fdef7dc-e355-4b27-9e2d-3fa8edfa2358</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -71596,7 +71640,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>4bd0d53d-77db-4f85-a8a0-1d81a2e2b949</t>
+          <t>e7da24d1-3207-4e89-b194-f8d0236ec5a5</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -71647,7 +71691,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>8488ccf0-20eb-436e-84ef-b5f12179e498</t>
+          <t>ceae9362-8ad9-47de-9dd7-5c7aab37c180</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -71698,7 +71742,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>0eeb4d7b-583e-436a-8758-454a071e55bf</t>
+          <t>aca39269-6cc6-49e7-9379-84ac2f1b5319</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -71749,7 +71793,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>abd0e436-199b-4e3c-a7a0-b27bbade7781</t>
+          <t>73632ff0-0465-4ee5-b567-a57ca593cbb1</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -71800,7 +71844,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>8f8942af-c930-4100-881a-e96a4f95983f</t>
+          <t>0f8072c3-b465-4eb0-96e6-c58020d671a2</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -71851,7 +71895,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>ff2ed429-0202-404e-8b5f-324e14bb4b6a</t>
+          <t>3c8d30d1-f6d8-493b-aaa6-de9fb8ea6f6a</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -71902,7 +71946,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>5cdd23ff-5089-45fc-b9cb-e1110a649f75</t>
+          <t>6e89b223-dd4d-427d-87c0-ba89a6f3de44</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -71953,7 +71997,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>534dd986-2da6-4dd4-a2ec-3f19cd7fbec1</t>
+          <t>bc5ea489-fda7-439f-8ecf-37b905105a45</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -72004,7 +72048,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>31d1dc70-4d42-4c2f-b3e8-1d0c3053ec5d</t>
+          <t>37798064-9f0b-45ec-affb-3a2124964d5b</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -72055,7 +72099,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>17b8aba4-52e3-455d-8c2d-0d62216096fe</t>
+          <t>b6f54fff-72a0-4dc1-86e9-6a9c7fbcf583</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -72106,7 +72150,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>1dc9389c-f4e6-4fb6-ba2b-6369a6382b54</t>
+          <t>94a86b17-0db6-4f63-8822-5b35ef04a967</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -72157,7 +72201,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>8d673311-c98b-444e-878a-814a55087583</t>
+          <t>557b9ea9-c670-4a09-a7b7-47aadd73a2d9</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -72208,7 +72252,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>ec0c0a25-2459-4227-bb0e-6aa2951d289b</t>
+          <t>ace7846c-37e6-4e8f-9200-75e1fb498751</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -72259,7 +72303,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>abf428eb-e881-426d-a6ab-fa5a9d224df2</t>
+          <t>c8d2e929-02c3-4ec0-8963-aabcaf6a1be8</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -72310,7 +72354,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>d57494c7-6350-4547-9b32-6e692b8c8e91</t>
+          <t>7cd6c2fe-5812-4aae-8711-a2fdb96ee20e</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -72361,7 +72405,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>49159b7c-f1ee-484b-bdfa-5a37856d6e3f</t>
+          <t>1edb8f43-bc7d-4014-ac59-c7184983ecf5</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -72412,7 +72456,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>ca434ee8-638f-41e1-b9d2-73a11cd4ce87</t>
+          <t>c4f1d998-7846-4775-aa46-445c23d12ca7</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -72463,7 +72507,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>c65e177a-671b-49e2-8108-8601ffbae1a3</t>
+          <t>329c5ad1-ea2e-49cd-9840-b45d20bb806b</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -72514,7 +72558,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>fcc5933e-49e6-4d59-930b-b94d8c7bd833</t>
+          <t>647aa381-4261-42c8-8776-21b2ac0572fd</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -72565,7 +72609,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>da2f8964-fd47-4987-b5c7-d1d87ed823e0</t>
+          <t>fe041b73-ba1e-4a67-a7c3-a1239477e371</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -72616,7 +72660,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>04c10bf3-7854-4f85-b0aa-eadb0c4014b6</t>
+          <t>b9045664-2558-4103-8346-0ea151de47f9</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -72667,7 +72711,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>dfa113d5-cf0c-45d7-ab77-8a1664130a63</t>
+          <t>4c73375b-1c1e-4a5b-b16d-51619916e690</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -72718,7 +72762,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>e2bc50ae-b88c-4503-aa4f-c5d2882b93ad</t>
+          <t>47a5afe8-18e7-4d0c-a139-47c5d911f169</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -72769,7 +72813,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>f7409aa9-8811-4292-ab1c-d8552a331482</t>
+          <t>b5eabe62-cd8c-475a-bec6-bebf81843c87</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -72820,7 +72864,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>3bf0de50-336f-4e9b-be0f-0a874f90bc8e</t>
+          <t>0fd1c34c-06a0-4379-8b13-8e3ce4f13940</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -72871,7 +72915,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>c3cba96f-6dbf-4d64-97ef-2ed1685445c0</t>
+          <t>c9ff500b-16df-4724-a403-559d0845dffd</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -72922,7 +72966,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2a355782-2cca-4ea6-909d-8e810eb7cea8</t>
+          <t>00325b54-e673-4821-826b-ab06bb74f491</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -72973,7 +73017,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>851215f4-6436-4332-9e32-693366e1c33d</t>
+          <t>b88a4239-4e4f-46fa-bb70-850aafc53119</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -73024,7 +73068,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>b83a40c4-ba8e-4010-8509-7c607834a571</t>
+          <t>eec28dc2-77b6-44b8-85af-24db77488baf</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -73075,7 +73119,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>cc2dd004-f746-4ebc-8b05-3ec8fb1537c0</t>
+          <t>91136890-8690-4237-82cf-e9d4dabff00e</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -73126,7 +73170,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>f763d3ef-d90e-44fc-937a-3f4a24a1fb6f</t>
+          <t>273cc011-8853-4a73-8998-eb9d0fba79e3</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -73177,7 +73221,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>f414166f-969f-45d7-9ac2-610218a03613</t>
+          <t>d4fa6429-d8b5-49b3-bde7-b70db9c8133e</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -73228,7 +73272,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>d7f5d3fc-cdb8-4fba-9f7f-72fb98a62977</t>
+          <t>d766735a-5140-4ca5-88ee-00660e5c6399</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -73279,7 +73323,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>f4502a34-aafa-459b-9db9-1262087907ec</t>
+          <t>04843650-49ab-4273-8899-e001b996f49d</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -73330,7 +73374,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>1c4ddc5d-9224-4d46-b20e-0f547d5b2175</t>
+          <t>27fc219e-16b6-4df0-8039-cf5f7fac198b</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -73381,7 +73425,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>927479fa-1228-4a71-ad77-1a68603e8978</t>
+          <t>b8a250de-e913-430d-8068-747ed91d67fb</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -73432,7 +73476,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>6456d93a-a2c7-4632-a056-d06d25715770</t>
+          <t>70698bc5-42e5-4074-94c4-65ee2106fb84</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -73483,7 +73527,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>cf2b59c3-0f33-4253-a7c2-758139738869</t>
+          <t>fd73f4b1-6518-4bcc-b515-60863e134ada</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -73534,7 +73578,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>f35e1c17-4711-442f-bdc1-6efc21e03dae</t>
+          <t>26824e02-63c3-4c5d-8e0a-273f3df690cd</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -73585,7 +73629,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>937ef8a7-4cf0-4db3-ba71-0c7e1a0ce944</t>
+          <t>19ae9a0b-6fc5-4f22-adb2-722e40162455</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -73636,7 +73680,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>d451aad2-8a10-4a2e-8277-a201b0488c90</t>
+          <t>fd2ade6e-46ae-498c-a537-f7312ff3ba9a</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -73687,7 +73731,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>333fcb62-c2a2-4478-98ef-467291a14323</t>
+          <t>a5e13a16-b9d4-450b-96f8-4967b3f8b123</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -73738,7 +73782,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>bc7f97aa-0a10-40ea-8b04-98269ba5173c</t>
+          <t>92c54a65-808b-41cf-9e4d-0b35ae57ac69</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -73789,7 +73833,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>0a23e5d2-8960-4b31-b504-14dc9190e5e8</t>
+          <t>83ebf73a-08a4-4a6a-862f-26fd02ee5489</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -73840,7 +73884,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>e349aafa-cf8b-47c3-9093-38435e0b5a44</t>
+          <t>9523965f-e9ab-49d6-8e77-90ef7b6c0eee</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -73891,7 +73935,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>90d19402-295a-4d3c-8c4f-f5bed5e03dba</t>
+          <t>5fa44d97-d447-49fe-9b0e-c990e56a23ba</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">

</xml_diff>

<commit_message>
Remove Availability History tab and clear availability requests from Excel
</commit_message>
<xml_diff>
--- a/api/backend/uploads/ibu_schedule.xlsx
+++ b/api/backend/uploads/ibu_schedule.xlsx
@@ -62787,7 +62787,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P96"/>
+  <dimension ref="A1:P1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -62870,4261 +62870,6 @@
         <is>
           <t>Approved_At</t>
         </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>5e350372-3873-45df-b4e0-5a0eaea0033f</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>emp_017</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>["wednesday"]</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K2" s="463" t="n">
-        <v>46182.68044114584</v>
-      </c>
-      <c r="N2" s="463" t="n">
-        <v>46182.68076206018</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>d1dce9f4-aeaf-4c66-8d31-76629b71dc2a</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>emp_012</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>["monday"]</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K3" s="463" t="n">
-        <v>46182.68198248842</v>
-      </c>
-      <c r="N3" s="463" t="n">
-        <v>46182.68348252315</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>81840131-cc5d-45f6-953b-dd1d3026dba8</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>emp_012</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>["tuesday"]</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K4" s="463" t="n">
-        <v>46182.68207266204</v>
-      </c>
-      <c r="N4" s="463" t="n">
-        <v>46182.68352160879</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>ed78e80a-1433-4cfe-a9f1-53b8c59c0efd</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>emp_012</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>["wednesday"]</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K5" s="463" t="n">
-        <v>46182.68215238426</v>
-      </c>
-      <c r="N5" s="463" t="n">
-        <v>46182.68356034722</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>506e7912-892f-41de-a323-0d49bf5d6cf3</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>emp_012</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>["thursday"]</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K6" s="463" t="n">
-        <v>46182.68222422454</v>
-      </c>
-      <c r="N6" s="463" t="n">
-        <v>46182.68359472222</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>94ea3630-6e99-4754-b87b-dac4cd239643</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>emp_012</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>["friday"]</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K7" s="463" t="n">
-        <v>46182.68230407407</v>
-      </c>
-      <c r="N7" s="463" t="n">
-        <v>46182.68363207176</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>246c0a1e-8160-4b55-a0c6-47e533956191</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>emp_012</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>["saturday"]</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K8" s="463" t="n">
-        <v>46182.68242398148</v>
-      </c>
-      <c r="N8" s="463" t="n">
-        <v>46182.6836652662</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>2525fb94-abbe-45ad-bca3-67748dbd04eb</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>emp_004</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>["monday"]</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K9" s="463" t="n">
-        <v>46182.68266236111</v>
-      </c>
-      <c r="N9" s="463" t="n">
-        <v>46182.68369596065</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>690d5ec8-9492-429e-87cd-22656df8669e</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>emp_008</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>["thursday"]</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K10" s="463" t="n">
-        <v>46182.68321407407</v>
-      </c>
-      <c r="N10" s="463" t="n">
-        <v>46182.68373296296</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>dade82cd-afbb-4d51-97ad-943def51a24f</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>emp_004</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>["tuesday"]</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K11" s="463" t="n">
-        <v>46182.68739420139</v>
-      </c>
-      <c r="N11" s="463" t="n">
-        <v>46182.69697668982</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>e5f65cc8-e3cc-45f8-afd2-1d97821506da</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>emp_004</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>["thursday"]</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K12" s="463" t="n">
-        <v>46182.68786140046</v>
-      </c>
-      <c r="N12" s="463" t="n">
-        <v>46182.69704689815</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>e5810a83-1be1-4ee2-a2a8-2a4c473ae2e0</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>emp_004</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>["friday"]</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K13" s="463" t="n">
-        <v>46182.68794916667</v>
-      </c>
-      <c r="N13" s="463" t="n">
-        <v>46182.69711325232</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>34900a54-60a1-4ffa-b2cf-19863578763e</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>emp_004</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>["saturday"]</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K14" s="463" t="n">
-        <v>46182.68812075232</v>
-      </c>
-      <c r="N14" s="463" t="n">
-        <v>46182.69716332176</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>6863fe2e-82a3-43ab-ab32-2b8dde9a3229</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>emp_005</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>["monday"]</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K15" s="463" t="n">
-        <v>46182.68837650463</v>
-      </c>
-      <c r="N15" s="463" t="n">
-        <v>46182.69721660879</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>153abfe4-9e80-410a-9808-13413eaaf50d</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>emp_005</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>["tuesday"]</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K16" s="463" t="n">
-        <v>46182.68843890046</v>
-      </c>
-      <c r="N16" s="463" t="n">
-        <v>46182.6972512963</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>cb120672-fbf3-4d0d-b12e-1c77362da959</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>emp_005</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>["wednesday"]</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K17" s="463" t="n">
-        <v>46182.68849805556</v>
-      </c>
-      <c r="N17" s="463" t="n">
-        <v>46182.69727876157</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>a74cacda-1ca1-4896-bc22-656a4d46e068</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>emp_005</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>["thursday"]</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K18" s="463" t="n">
-        <v>46182.68856417824</v>
-      </c>
-      <c r="N18" s="463" t="n">
-        <v>46182.69732396991</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>b13db310-e544-439a-933b-270278ba33be</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>emp_005</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>["friday"]</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K19" s="463" t="n">
-        <v>46182.68863230324</v>
-      </c>
-      <c r="N19" s="463" t="n">
-        <v>46182.6974062037</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>7c975e00-a489-4afa-93e4-5d45c2ce3830</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>emp_005</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>["saturday"]</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K20" s="463" t="n">
-        <v>46182.69046516204</v>
-      </c>
-      <c r="N20" s="463" t="n">
-        <v>46182.69744298611</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>dd79bdfd-24c2-43ed-85bb-e4ffd49d3230</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>emp_006</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>["wednesday"]</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K21" s="463" t="n">
-        <v>46182.69069785879</v>
-      </c>
-      <c r="N21" s="463" t="n">
-        <v>46182.69749107639</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>406222ed-a8f1-4df9-b5ba-c625f86027ad</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>emp_006</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>["thursday"]</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K22" s="463" t="n">
-        <v>46182.69120728009</v>
-      </c>
-      <c r="N22" s="463" t="n">
-        <v>46182.69752792824</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>59594dbe-8e35-418e-9066-17845309f975</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>emp_007</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>["monday"]</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K23" s="463" t="n">
-        <v>46182.69168170139</v>
-      </c>
-      <c r="N23" s="463" t="n">
-        <v>46182.69757763889</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>90f7067c-3e66-4218-8a9c-476a40604f10</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>emp_007</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>["tuesday"]</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K24" s="463" t="n">
-        <v>46182.6917419676</v>
-      </c>
-      <c r="N24" s="463" t="n">
-        <v>46182.69762542824</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>5bc1ac82-6e3d-4d74-b8b5-f1586c76b75e</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>emp_007</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>["wednesday"]</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K25" s="463" t="n">
-        <v>46182.6918153125</v>
-      </c>
-      <c r="N25" s="463" t="n">
-        <v>46182.69766206019</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>194399ea-47ea-4b79-9975-2f949ccb9a88</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>emp_007</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>["thursday"]</t>
-        </is>
-      </c>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K26" s="463" t="n">
-        <v>46182.69189060185</v>
-      </c>
-      <c r="N26" s="463" t="n">
-        <v>46182.69769990741</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>1f758ca0-850b-47e9-9951-b13f93c201a7</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>emp_007</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>["wednesday"]</t>
-        </is>
-      </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K27" s="463" t="n">
-        <v>46182.69198528936</v>
-      </c>
-      <c r="N27" s="463" t="n">
-        <v>46182.69777811343</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>b6b1c7fc-d571-4a46-ae59-bb255c576cf8</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>emp_007</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>["friday"]</t>
-        </is>
-      </c>
-      <c r="I28" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K28" s="463" t="n">
-        <v>46182.6920941088</v>
-      </c>
-      <c r="N28" s="463" t="n">
-        <v>46182.69785590278</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>509991c1-4cce-4b30-9af7-c728f723a9f3</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>emp_008</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>["tuesday"]</t>
-        </is>
-      </c>
-      <c r="I29" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K29" s="463" t="n">
-        <v>46182.69242583333</v>
-      </c>
-      <c r="N29" s="463" t="n">
-        <v>46182.69790143518</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>eaa6b272-c001-4376-a096-fd5d3b4b7857</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>emp_008</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>["friday"]</t>
-        </is>
-      </c>
-      <c r="I30" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K30" s="463" t="n">
-        <v>46182.69258614584</v>
-      </c>
-      <c r="N30" s="463" t="n">
-        <v>46182.69797137732</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>9a284d4e-0aa3-405a-b470-3f6907995eb0</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>emp_009</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>["monday"]</t>
-        </is>
-      </c>
-      <c r="I31" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K31" s="463" t="n">
-        <v>46182.69281082176</v>
-      </c>
-      <c r="N31" s="463" t="n">
-        <v>46182.69800782407</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>80b26006-ef7c-43c2-8921-c4b9a55fca29</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>emp_009</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>["tuesday"]</t>
-        </is>
-      </c>
-      <c r="I32" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K32" s="463" t="n">
-        <v>46182.69289650463</v>
-      </c>
-      <c r="N32" s="463" t="n">
-        <v>46182.69808212963</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>38d7e008-b497-4adf-879e-4bcff9b4cae2</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>emp_009</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>["thursday"]</t>
-        </is>
-      </c>
-      <c r="I33" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K33" s="463" t="n">
-        <v>46182.69300927084</v>
-      </c>
-      <c r="N33" s="463" t="n">
-        <v>46182.69812122685</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>6b9bb626-1e77-4857-b409-45a50555a13e</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>emp_009</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>["friday"]</t>
-        </is>
-      </c>
-      <c r="I34" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K34" s="463" t="n">
-        <v>46182.69309910879</v>
-      </c>
-      <c r="N34" s="463" t="n">
-        <v>46182.69816709491</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>d200b466-ea59-4a12-bb36-38e417e1852d</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>emp_010</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>["thursday"]</t>
-        </is>
-      </c>
-      <c r="I35" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K35" s="463" t="n">
-        <v>46182.69325486111</v>
-      </c>
-      <c r="N35" s="463" t="n">
-        <v>46182.69824834491</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>4923902c-3635-4c8e-afdc-ad94e2d54c11</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>emp_011</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>["monday"]</t>
-        </is>
-      </c>
-      <c r="I36" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K36" s="463" t="n">
-        <v>46182.69348269676</v>
-      </c>
-      <c r="N36" s="463" t="n">
-        <v>46182.6982859838</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>ce69916f-291b-4cf6-9c5b-54f01beffd8b</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>emp_011</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>["tuesday"]</t>
-        </is>
-      </c>
-      <c r="I37" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K37" s="463" t="n">
-        <v>46182.69357153935</v>
-      </c>
-      <c r="N37" s="463" t="n">
-        <v>46182.69832219907</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>c17dd068-deca-441a-be40-82369a4abc5a</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>emp_011</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>["wednesday"]</t>
-        </is>
-      </c>
-      <c r="I38" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K38" s="463" t="n">
-        <v>46182.69362791667</v>
-      </c>
-      <c r="N38" s="463" t="n">
-        <v>46182.69840618056</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>d9487943-47a2-4536-800b-518fb76a2544</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>emp_011</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>["thursday"]</t>
-        </is>
-      </c>
-      <c r="I39" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K39" s="463" t="n">
-        <v>46182.69368649305</v>
-      </c>
-      <c r="N39" s="463" t="n">
-        <v>46182.69845453704</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>e227e662-7ebb-4cb3-a96f-bf497c7d0282</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>emp_011</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>["friday"]</t>
-        </is>
-      </c>
-      <c r="I40" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K40" s="463" t="n">
-        <v>46182.69375005787</v>
-      </c>
-      <c r="N40" s="463" t="n">
-        <v>46182.69914417824</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>2d11ada0-d48b-4e49-af01-fd9b8953bb96</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>emp_011</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>["saturday"]</t>
-        </is>
-      </c>
-      <c r="I41" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K41" s="463" t="n">
-        <v>46182.69384526621</v>
-      </c>
-      <c r="N41" s="463" t="n">
-        <v>46182.69849435185</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>80cb8f57-b89e-4c22-b4c5-ca49e262487c</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>emp_013</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>["monday"]</t>
-        </is>
-      </c>
-      <c r="I42" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K42" s="463" t="n">
-        <v>46182.69419137731</v>
-      </c>
-      <c r="N42" s="463" t="n">
-        <v>46182.69856702547</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>43d72d48-3ba6-4fa8-b87c-c94d22ae2ba2</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>emp_013</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>["tuesday"]</t>
-        </is>
-      </c>
-      <c r="I43" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K43" s="463" t="n">
-        <v>46182.69425256945</v>
-      </c>
-      <c r="N43" s="463" t="n">
-        <v>46182.69853018518</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>eae4c465-13cb-4f3f-b8fb-f2b48b21a5ad</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>emp_013</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F44" t="inlineStr">
-        <is>
-          <t>["wednesday"]</t>
-        </is>
-      </c>
-      <c r="I44" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K44" s="463" t="n">
-        <v>46182.69434773148</v>
-      </c>
-      <c r="N44" s="463" t="n">
-        <v>46182.69860277777</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>6b885407-4dd8-40c4-81b8-c8251d2bc4ce</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>emp_013</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>["thursday"]</t>
-        </is>
-      </c>
-      <c r="I45" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K45" s="463" t="n">
-        <v>46182.69459594908</v>
-      </c>
-      <c r="N45" s="463" t="n">
-        <v>46182.69863982639</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>fc4dd01a-d6de-4d5d-ae93-abf2d0c7e4a3</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>emp_013</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>["friday"]</t>
-        </is>
-      </c>
-      <c r="I46" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K46" s="463" t="n">
-        <v>46182.69467006945</v>
-      </c>
-      <c r="N46" s="463" t="n">
-        <v>46182.69867885417</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>a1835ac8-1d24-40bd-a0f1-59b0f4c4e400</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>emp_013</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>["saturday"]</t>
-        </is>
-      </c>
-      <c r="I47" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K47" s="463" t="n">
-        <v>46182.69473725694</v>
-      </c>
-      <c r="N47" s="463" t="n">
-        <v>46182.69872133102</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>582a4323-f554-4940-95fa-3449dc12b323</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>emp_011</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F48" t="inlineStr">
-        <is>
-          <t>["monday"]</t>
-        </is>
-      </c>
-      <c r="I48" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K48" s="463" t="n">
-        <v>46182.69500721065</v>
-      </c>
-      <c r="N48" s="463" t="n">
-        <v>46182.69875952546</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>741e7249-8ca6-47f9-87f6-1fd00d6d6e0c</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>emp_014</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>["tuesday"]</t>
-        </is>
-      </c>
-      <c r="I49" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K49" s="463" t="n">
-        <v>46182.69524296296</v>
-      </c>
-      <c r="N49" s="463" t="n">
-        <v>46182.69879672454</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>a3103d37-e7f0-4645-8174-1ad03c43cdc4</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>emp_015</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>["monday"]</t>
-        </is>
-      </c>
-      <c r="I50" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K50" s="463" t="n">
-        <v>46182.69542989583</v>
-      </c>
-      <c r="N50" s="463" t="n">
-        <v>46182.69887462963</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>3545e125-9a8e-4112-b4e8-6a688228f9d1</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>emp_015</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>["thursday"]</t>
-        </is>
-      </c>
-      <c r="I51" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K51" s="463" t="n">
-        <v>46182.69551966435</v>
-      </c>
-      <c r="N51" s="463" t="n">
-        <v>46182.69892596065</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>fa48b653-7ac2-4931-ba72-fea9a41fa993</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>emp_015</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t>["saturday"]</t>
-        </is>
-      </c>
-      <c r="I52" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K52" s="463" t="n">
-        <v>46182.69561778935</v>
-      </c>
-      <c r="N52" s="463" t="n">
-        <v>46182.69901015046</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>25c30fba-7e12-446e-95db-41998ad5c376</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>emp_016</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F53" t="inlineStr">
-        <is>
-          <t>["tuesday"]</t>
-        </is>
-      </c>
-      <c r="I53" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K53" s="463" t="n">
-        <v>46182.6959509838</v>
-      </c>
-      <c r="N53" s="463" t="n">
-        <v>46182.69905035879</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>4e33c437-46ed-4e3d-9a9a-b2b617a36899</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>emp_016</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F54" t="inlineStr">
-        <is>
-          <t>["thursday"]</t>
-        </is>
-      </c>
-      <c r="I54" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K54" s="463" t="n">
-        <v>46182.69604675926</v>
-      </c>
-      <c r="N54" s="463" t="n">
-        <v>46182.69909200232</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>e9a0e2b9-c4dd-4937-800c-7052d82c85db</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>emp_011</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F55" t="inlineStr">
-        <is>
-          <t>["monday"]</t>
-        </is>
-      </c>
-      <c r="I55" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K55" s="463" t="n">
-        <v>46182.70189392361</v>
-      </c>
-      <c r="N55" s="463" t="n">
-        <v>46182.7082630787</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>72caa2e8-d976-47c6-a545-aea1e29e8330</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>emp_011</t>
-        </is>
-      </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F56" t="inlineStr">
-        <is>
-          <t>["tuesday"]</t>
-        </is>
-      </c>
-      <c r="I56" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K56" s="463" t="n">
-        <v>46182.70203262731</v>
-      </c>
-      <c r="N56" s="463" t="n">
-        <v>46182.70830813657</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>a252f2f1-4803-46cf-9998-eaf68f256830</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>emp_011</t>
-        </is>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E57" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F57" t="inlineStr">
-        <is>
-          <t>["wednesday"]</t>
-        </is>
-      </c>
-      <c r="I57" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K57" s="463" t="n">
-        <v>46182.70209701389</v>
-      </c>
-      <c r="N57" s="463" t="n">
-        <v>46182.70944013889</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>5b01f049-35fd-45f9-ad2b-de242d9cb875</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>emp_011</t>
-        </is>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E58" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F58" t="inlineStr">
-        <is>
-          <t>["thursday"]</t>
-        </is>
-      </c>
-      <c r="I58" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K58" s="463" t="n">
-        <v>46182.70215707176</v>
-      </c>
-      <c r="N58" s="463" t="n">
-        <v>46182.7094005787</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>e33cf1b9-f51a-44b7-a4e6-2e1cc63cbc61</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>emp_011</t>
-        </is>
-      </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F59" t="inlineStr">
-        <is>
-          <t>["friday"]</t>
-        </is>
-      </c>
-      <c r="I59" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K59" s="463" t="n">
-        <v>46182.70221800926</v>
-      </c>
-      <c r="N59" s="463" t="n">
-        <v>46182.70835635417</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>07ae7b22-b55d-43e3-abcc-85743bda175d</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>emp_005</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D60" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E60" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F60" t="inlineStr">
-        <is>
-          <t>["monday"]</t>
-        </is>
-      </c>
-      <c r="I60" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K60" s="463" t="n">
-        <v>46182.70277211806</v>
-      </c>
-      <c r="N60" s="463" t="n">
-        <v>46182.70839515046</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>17ffb497-0178-479a-86af-131e9a26023d</t>
-        </is>
-      </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>emp_005</t>
-        </is>
-      </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E61" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F61" t="inlineStr">
-        <is>
-          <t>["tuesday"]</t>
-        </is>
-      </c>
-      <c r="I61" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K61" s="463" t="n">
-        <v>46182.70299961806</v>
-      </c>
-      <c r="N61" s="463" t="n">
-        <v>46182.70843331019</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>5e02758b-8548-473a-81f9-a10b70e20326</t>
-        </is>
-      </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>emp_005</t>
-        </is>
-      </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D62" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E62" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F62" t="inlineStr">
-        <is>
-          <t>["wednesday"]</t>
-        </is>
-      </c>
-      <c r="I62" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K62" s="463" t="n">
-        <v>46182.70317165509</v>
-      </c>
-      <c r="N62" s="463" t="n">
-        <v>46182.70847239583</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>9e16dfb1-01ca-416c-9d33-09a0694210bc</t>
-        </is>
-      </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>emp_005</t>
-        </is>
-      </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F63" t="inlineStr">
-        <is>
-          <t>["thursday"]</t>
-        </is>
-      </c>
-      <c r="I63" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K63" s="463" t="n">
-        <v>46182.7033025463</v>
-      </c>
-      <c r="N63" s="463" t="n">
-        <v>46182.70851172454</v>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>4c9fc6ad-f0b5-4ad1-9dfd-521c4113cb49</t>
-        </is>
-      </c>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>emp_005</t>
-        </is>
-      </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D64" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E64" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F64" t="inlineStr">
-        <is>
-          <t>["friday"]</t>
-        </is>
-      </c>
-      <c r="I64" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K64" s="463" t="n">
-        <v>46182.70341662037</v>
-      </c>
-      <c r="N64" s="463" t="n">
-        <v>46182.70854988426</v>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>fbadfb3e-8cca-47bd-b5ef-d505c6eb7f4e</t>
-        </is>
-      </c>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t>emp_004</t>
-        </is>
-      </c>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D65" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E65" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F65" t="inlineStr">
-        <is>
-          <t>["monday"]</t>
-        </is>
-      </c>
-      <c r="I65" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K65" s="463" t="n">
-        <v>46182.70396266204</v>
-      </c>
-      <c r="N65" s="463" t="n">
-        <v>46182.70858949074</v>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>cd16ff12-6d9a-4f73-8883-7547766e9b29</t>
-        </is>
-      </c>
-      <c r="B66" t="inlineStr">
-        <is>
-          <t>emp_004</t>
-        </is>
-      </c>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D66" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E66" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F66" t="inlineStr">
-        <is>
-          <t>["tuesday"]</t>
-        </is>
-      </c>
-      <c r="I66" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K66" s="463" t="n">
-        <v>46182.70407003472</v>
-      </c>
-      <c r="N66" s="463" t="n">
-        <v>46182.70862930555</v>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t>1390715d-fed4-4e57-8ffa-571b3a0670c2</t>
-        </is>
-      </c>
-      <c r="B67" t="inlineStr">
-        <is>
-          <t>emp_004</t>
-        </is>
-      </c>
-      <c r="C67" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D67" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E67" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F67" t="inlineStr">
-        <is>
-          <t>["wednesday"]</t>
-        </is>
-      </c>
-      <c r="I67" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K67" s="463" t="n">
-        <v>46182.70417866898</v>
-      </c>
-      <c r="N67" s="463" t="n">
-        <v>46182.70866736111</v>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" t="inlineStr">
-        <is>
-          <t>ccab1686-b42c-4023-bf7d-a5f93a0f18f8</t>
-        </is>
-      </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>emp_004</t>
-        </is>
-      </c>
-      <c r="C68" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D68" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E68" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F68" t="inlineStr">
-        <is>
-          <t>["thursday"]</t>
-        </is>
-      </c>
-      <c r="I68" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K68" s="463" t="n">
-        <v>46182.70427731481</v>
-      </c>
-      <c r="N68" s="463" t="n">
-        <v>46182.70870700231</v>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" t="inlineStr">
-        <is>
-          <t>08cb9dca-6dbd-4af8-8240-47f6449acdd8</t>
-        </is>
-      </c>
-      <c r="B69" t="inlineStr">
-        <is>
-          <t>emp_004</t>
-        </is>
-      </c>
-      <c r="C69" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D69" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E69" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F69" t="inlineStr">
-        <is>
-          <t>["friday"]</t>
-        </is>
-      </c>
-      <c r="I69" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K69" s="463" t="n">
-        <v>46182.70437729167</v>
-      </c>
-      <c r="N69" s="463" t="n">
-        <v>46182.70874456019</v>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" t="inlineStr">
-        <is>
-          <t>74080ff0-ebc6-4d7e-8a30-b3b3ec5ea1ea</t>
-        </is>
-      </c>
-      <c r="B70" t="inlineStr">
-        <is>
-          <t>emp_006</t>
-        </is>
-      </c>
-      <c r="C70" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D70" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E70" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F70" t="inlineStr">
-        <is>
-          <t>["monday"]</t>
-        </is>
-      </c>
-      <c r="I70" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K70" s="463" t="n">
-        <v>46182.70497670139</v>
-      </c>
-      <c r="N70" s="463" t="n">
-        <v>46182.70878143518</v>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t>27da64b6-3dd0-423b-b1de-f2246a2dea11</t>
-        </is>
-      </c>
-      <c r="B71" t="inlineStr">
-        <is>
-          <t>emp_006</t>
-        </is>
-      </c>
-      <c r="C71" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D71" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E71" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F71" t="inlineStr">
-        <is>
-          <t>["tuesday"]</t>
-        </is>
-      </c>
-      <c r="I71" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K71" s="463" t="n">
-        <v>46182.70507425926</v>
-      </c>
-      <c r="N71" s="463" t="n">
-        <v>46182.70882163195</v>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" t="inlineStr">
-        <is>
-          <t>0873bef1-2040-4d65-a150-21f029d98d82</t>
-        </is>
-      </c>
-      <c r="B72" t="inlineStr">
-        <is>
-          <t>emp_006</t>
-        </is>
-      </c>
-      <c r="C72" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D72" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E72" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F72" t="inlineStr">
-        <is>
-          <t>["wednesday"]</t>
-        </is>
-      </c>
-      <c r="I72" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K72" s="463" t="n">
-        <v>46182.70517010416</v>
-      </c>
-      <c r="N72" s="463" t="n">
-        <v>46182.70886113426</v>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" t="inlineStr">
-        <is>
-          <t>1b8e907b-f433-4539-9bdc-c6da15d3d6a6</t>
-        </is>
-      </c>
-      <c r="B73" t="inlineStr">
-        <is>
-          <t>emp_006</t>
-        </is>
-      </c>
-      <c r="C73" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D73" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E73" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F73" t="inlineStr">
-        <is>
-          <t>["thursday"]</t>
-        </is>
-      </c>
-      <c r="I73" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K73" s="463" t="n">
-        <v>46182.70539097222</v>
-      </c>
-      <c r="N73" s="463" t="n">
-        <v>46182.70890368056</v>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" t="inlineStr">
-        <is>
-          <t>b40802f7-755b-4ce7-911d-eee41d15e9b1</t>
-        </is>
-      </c>
-      <c r="B74" t="inlineStr">
-        <is>
-          <t>emp_006</t>
-        </is>
-      </c>
-      <c r="C74" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D74" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E74" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F74" t="inlineStr">
-        <is>
-          <t>["friday"]</t>
-        </is>
-      </c>
-      <c r="I74" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K74" s="463" t="n">
-        <v>46182.70549178241</v>
-      </c>
-      <c r="N74" s="463" t="n">
-        <v>46182.70894511574</v>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" t="inlineStr">
-        <is>
-          <t>881c9fc1-9ed0-48c2-b756-68bc09da69b4</t>
-        </is>
-      </c>
-      <c r="B75" t="inlineStr">
-        <is>
-          <t>emp_013</t>
-        </is>
-      </c>
-      <c r="C75" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D75" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E75" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F75" t="inlineStr">
-        <is>
-          <t>["monday"]</t>
-        </is>
-      </c>
-      <c r="I75" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K75" s="463" t="n">
-        <v>46182.70635791666</v>
-      </c>
-      <c r="N75" s="463" t="n">
-        <v>46182.70898407407</v>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" t="inlineStr">
-        <is>
-          <t>b01959e8-2432-43a1-b478-77e93d2c1b0c</t>
-        </is>
-      </c>
-      <c r="B76" t="inlineStr">
-        <is>
-          <t>emp_013</t>
-        </is>
-      </c>
-      <c r="C76" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D76" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E76" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F76" t="inlineStr">
-        <is>
-          <t>["tuesday"]</t>
-        </is>
-      </c>
-      <c r="I76" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K76" s="463" t="n">
-        <v>46182.70646814815</v>
-      </c>
-      <c r="N76" s="463" t="n">
-        <v>46182.70903457176</v>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" t="inlineStr">
-        <is>
-          <t>123a3cbd-fc2c-4d61-8027-d98be3e0111e</t>
-        </is>
-      </c>
-      <c r="B77" t="inlineStr">
-        <is>
-          <t>emp_013</t>
-        </is>
-      </c>
-      <c r="C77" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D77" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E77" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F77" t="inlineStr">
-        <is>
-          <t>["wednesday"]</t>
-        </is>
-      </c>
-      <c r="I77" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K77" s="463" t="n">
-        <v>46182.70656483796</v>
-      </c>
-      <c r="N77" s="463" t="n">
-        <v>46182.70910758102</v>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" t="inlineStr">
-        <is>
-          <t>088132a6-5cfb-4a25-8e39-c3e4f67a6d0f</t>
-        </is>
-      </c>
-      <c r="B78" t="inlineStr">
-        <is>
-          <t>emp_013</t>
-        </is>
-      </c>
-      <c r="C78" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D78" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E78" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F78" t="inlineStr">
-        <is>
-          <t>["thursday"]</t>
-        </is>
-      </c>
-      <c r="I78" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K78" s="463" t="n">
-        <v>46182.70668165509</v>
-      </c>
-      <c r="N78" s="463" t="n">
-        <v>46182.70914438657</v>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" t="inlineStr">
-        <is>
-          <t>da409132-77bc-46e8-b4e3-29a3949e7374</t>
-        </is>
-      </c>
-      <c r="B79" t="inlineStr">
-        <is>
-          <t>emp_014</t>
-        </is>
-      </c>
-      <c r="C79" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D79" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E79" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F79" t="inlineStr">
-        <is>
-          <t>["monday"]</t>
-        </is>
-      </c>
-      <c r="I79" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K79" s="463" t="n">
-        <v>46182.70719875</v>
-      </c>
-      <c r="N79" s="463" t="n">
-        <v>46182.70918405092</v>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" t="inlineStr">
-        <is>
-          <t>7dfb9001-d92e-4e19-b3e2-65c291dc2c8e</t>
-        </is>
-      </c>
-      <c r="B80" t="inlineStr">
-        <is>
-          <t>emp_014</t>
-        </is>
-      </c>
-      <c r="C80" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D80" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E80" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F80" t="inlineStr">
-        <is>
-          <t>["tuesday"]</t>
-        </is>
-      </c>
-      <c r="I80" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K80" s="463" t="n">
-        <v>46182.70731101852</v>
-      </c>
-      <c r="N80" s="463" t="n">
-        <v>46182.70923268519</v>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" t="inlineStr">
-        <is>
-          <t>286243d0-2d41-4b5f-bab2-947f7395485f</t>
-        </is>
-      </c>
-      <c r="B81" t="inlineStr">
-        <is>
-          <t>emp_014</t>
-        </is>
-      </c>
-      <c r="C81" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D81" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E81" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F81" t="inlineStr">
-        <is>
-          <t>["wednesday"]</t>
-        </is>
-      </c>
-      <c r="I81" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K81" s="463" t="n">
-        <v>46182.70741693287</v>
-      </c>
-      <c r="N81" s="463" t="n">
-        <v>46182.70927535879</v>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" t="inlineStr">
-        <is>
-          <t>51491fea-7ef2-4224-9ce5-3824b29756a4</t>
-        </is>
-      </c>
-      <c r="B82" t="inlineStr">
-        <is>
-          <t>emp_014</t>
-        </is>
-      </c>
-      <c r="C82" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D82" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E82" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F82" t="inlineStr">
-        <is>
-          <t>["thursday"]</t>
-        </is>
-      </c>
-      <c r="I82" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K82" s="463" t="n">
-        <v>46182.70751994213</v>
-      </c>
-      <c r="N82" s="463" t="n">
-        <v>46182.70931619213</v>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" t="inlineStr">
-        <is>
-          <t>69be61f8-4060-4e7f-ae55-ed58ff5e22e3</t>
-        </is>
-      </c>
-      <c r="B83" t="inlineStr">
-        <is>
-          <t>emp_014</t>
-        </is>
-      </c>
-      <c r="C83" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D83" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E83" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F83" t="inlineStr">
-        <is>
-          <t>["friday"]</t>
-        </is>
-      </c>
-      <c r="I83" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K83" s="463" t="n">
-        <v>46182.70761918982</v>
-      </c>
-      <c r="N83" s="463" t="n">
-        <v>46182.70934950231</v>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" t="inlineStr">
-        <is>
-          <t>1f1361c6-3832-447b-88fc-fcbf085c15ab</t>
-        </is>
-      </c>
-      <c r="B84" t="inlineStr">
-        <is>
-          <t>emp_1781043065177</t>
-        </is>
-      </c>
-      <c r="C84" t="inlineStr">
-        <is>
-          <t>day_off</t>
-        </is>
-      </c>
-      <c r="D84" t="inlineStr">
-        <is>
-          <t>2026-06-09</t>
-        </is>
-      </c>
-      <c r="E84" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="F84" t="inlineStr">
-        <is>
-          <t>["monday"]</t>
-        </is>
-      </c>
-      <c r="I84" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.REJECTED</t>
-        </is>
-      </c>
-      <c r="J84" t="inlineStr">
-        <is>
-          <t>Sorry.</t>
-        </is>
-      </c>
-      <c r="M84" s="463" t="n">
-        <v>46182.78526831019</v>
-      </c>
-      <c r="N84" s="463" t="n">
-        <v>46182.80566619213</v>
-      </c>
-    </row>
-    <row r="85">
-      <c r="A85" t="inlineStr">
-        <is>
-          <t>0a972fd3-a970-47cf-b2a0-f5833edfd4d6</t>
-        </is>
-      </c>
-      <c r="B85" t="inlineStr">
-        <is>
-          <t>emp_1781043065177</t>
-        </is>
-      </c>
-      <c r="C85" t="inlineStr">
-        <is>
-          <t>day_off</t>
-        </is>
-      </c>
-      <c r="D85" t="inlineStr">
-        <is>
-          <t>2026-06-23</t>
-        </is>
-      </c>
-      <c r="E85" t="inlineStr">
-        <is>
-          <t>2026-06-23</t>
-        </is>
-      </c>
-      <c r="F85" t="inlineStr">
-        <is>
-          <t>["wednesday"]</t>
-        </is>
-      </c>
-      <c r="I85" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.REJECTED</t>
-        </is>
-      </c>
-      <c r="J85" t="inlineStr">
-        <is>
-          <t>s</t>
-        </is>
-      </c>
-      <c r="K85" t="inlineStr">
-        <is>
-          <t>Please approve.</t>
-        </is>
-      </c>
-      <c r="M85" s="463" t="n">
-        <v>46182.78545583333</v>
-      </c>
-      <c r="N85" s="463" t="n">
-        <v>46182.80940729166</v>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" t="inlineStr">
-        <is>
-          <t>666e44a8-8e15-4ed4-9591-9eda49744c49</t>
-        </is>
-      </c>
-      <c r="B86" t="inlineStr">
-        <is>
-          <t>emp_1781043065177</t>
-        </is>
-      </c>
-      <c r="C86" t="inlineStr">
-        <is>
-          <t>day_off</t>
-        </is>
-      </c>
-      <c r="D86" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E86" t="inlineStr">
-        <is>
-          <t>2026-06-22</t>
-        </is>
-      </c>
-      <c r="F86" t="inlineStr">
-        <is>
-          <t>["monday"]</t>
-        </is>
-      </c>
-      <c r="I86" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="M86" s="463" t="n">
-        <v>46182.78808515046</v>
-      </c>
-      <c r="N86" s="463" t="n">
-        <v>46182.80754699074</v>
-      </c>
-      <c r="O86" t="inlineStr">
-        <is>
-          <t>emp_1780946033840</t>
-        </is>
-      </c>
-      <c r="P86" s="463" t="n">
-        <v>46182.80754699074</v>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" t="inlineStr">
-        <is>
-          <t>a96dd354-5a74-48f9-a5ac-14b291a6f978</t>
-        </is>
-      </c>
-      <c r="B87" t="inlineStr">
-        <is>
-          <t>emp_1781043065177</t>
-        </is>
-      </c>
-      <c r="C87" t="inlineStr">
-        <is>
-          <t>day_off</t>
-        </is>
-      </c>
-      <c r="D87" t="inlineStr">
-        <is>
-          <t>2026-06-18</t>
-        </is>
-      </c>
-      <c r="E87" t="inlineStr">
-        <is>
-          <t>2026-06-18</t>
-        </is>
-      </c>
-      <c r="F87" t="inlineStr">
-        <is>
-          <t>["friday"]</t>
-        </is>
-      </c>
-      <c r="I87" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K87" t="inlineStr">
-        <is>
-          <t>Please approve.</t>
-        </is>
-      </c>
-      <c r="M87" s="463" t="n">
-        <v>46182.78831321759</v>
-      </c>
-      <c r="N87" s="463" t="n">
-        <v>46182.80759497685</v>
-      </c>
-      <c r="O87" t="inlineStr">
-        <is>
-          <t>emp_1780946033840</t>
-        </is>
-      </c>
-      <c r="P87" s="463" t="n">
-        <v>46182.80759497685</v>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" t="inlineStr">
-        <is>
-          <t>5f7d66fd-0994-478b-ad9b-e3a43d7c73fa</t>
-        </is>
-      </c>
-      <c r="B88" t="inlineStr">
-        <is>
-          <t>emp_1781043065177</t>
-        </is>
-      </c>
-      <c r="C88" t="inlineStr">
-        <is>
-          <t>day_off</t>
-        </is>
-      </c>
-      <c r="D88" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E88" t="inlineStr">
-        <is>
-          <t>2026-06-22</t>
-        </is>
-      </c>
-      <c r="F88" t="inlineStr">
-        <is>
-          <t>["monday"]</t>
-        </is>
-      </c>
-      <c r="I88" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K88" t="inlineStr">
-        <is>
-          <t>Approve boss.</t>
-        </is>
-      </c>
-      <c r="M88" s="463" t="n">
-        <v>46182.80669766204</v>
-      </c>
-      <c r="N88" s="463" t="n">
-        <v>46182.80763089121</v>
-      </c>
-      <c r="O88" t="inlineStr">
-        <is>
-          <t>emp_1780946033840</t>
-        </is>
-      </c>
-      <c r="P88" s="463" t="n">
-        <v>46182.80763089121</v>
-      </c>
-    </row>
-    <row r="89">
-      <c r="A89" t="inlineStr">
-        <is>
-          <t>5b018a26-b30c-4096-8800-a408ae2e1ec5</t>
-        </is>
-      </c>
-      <c r="B89" t="inlineStr">
-        <is>
-          <t>emp_1781043065177</t>
-        </is>
-      </c>
-      <c r="C89" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D89" t="inlineStr">
-        <is>
-          <t>2026-06-10</t>
-        </is>
-      </c>
-      <c r="E89" t="inlineStr">
-        <is>
-          <t>2026-06-26</t>
-        </is>
-      </c>
-      <c r="F89" t="inlineStr">
-        <is>
-          <t>["tuesday"]</t>
-        </is>
-      </c>
-      <c r="G89" t="inlineStr">
-        <is>
-          <t>08:00</t>
-        </is>
-      </c>
-      <c r="H89" t="inlineStr">
-        <is>
-          <t>09:00</t>
-        </is>
-      </c>
-      <c r="I89" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="J89" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="K89" t="inlineStr">
-        <is>
-          <t>Approve boss.</t>
-        </is>
-      </c>
-      <c r="M89" s="463" t="n">
-        <v>46182.80669996528</v>
-      </c>
-      <c r="N89" s="463" t="n">
-        <v>46182.80732481481</v>
-      </c>
-      <c r="O89" t="inlineStr">
-        <is>
-          <t>emp_1780946033840</t>
-        </is>
-      </c>
-      <c r="P89" s="463" t="n">
-        <v>46182.80732481481</v>
-      </c>
-    </row>
-    <row r="90">
-      <c r="A90" t="inlineStr">
-        <is>
-          <t>18c13503-ccac-4829-bf54-b3a5a943ead5</t>
-        </is>
-      </c>
-      <c r="B90" t="inlineStr">
-        <is>
-          <t>emp_1781043065177</t>
-        </is>
-      </c>
-      <c r="C90" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D90" t="inlineStr">
-        <is>
-          <t>2026-06-16</t>
-        </is>
-      </c>
-      <c r="E90" t="inlineStr">
-        <is>
-          <t>2026-06-26</t>
-        </is>
-      </c>
-      <c r="F90" t="inlineStr">
-        <is>
-          <t>["wednesday"]</t>
-        </is>
-      </c>
-      <c r="G90" t="inlineStr">
-        <is>
-          <t>12:00</t>
-        </is>
-      </c>
-      <c r="H90" t="inlineStr">
-        <is>
-          <t>17:00</t>
-        </is>
-      </c>
-      <c r="I90" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K90" t="inlineStr">
-        <is>
-          <t>Approve boss.</t>
-        </is>
-      </c>
-      <c r="M90" s="463" t="n">
-        <v>46182.80670422454</v>
-      </c>
-      <c r="N90" s="463" t="n">
-        <v>46182.80767947916</v>
-      </c>
-      <c r="O90" t="inlineStr">
-        <is>
-          <t>emp_1780946033840</t>
-        </is>
-      </c>
-      <c r="P90" s="463" t="n">
-        <v>46182.80767947916</v>
-      </c>
-    </row>
-    <row r="91">
-      <c r="A91" t="inlineStr">
-        <is>
-          <t>a5f2092e-9afe-45e5-89f2-7b90194ac3b4</t>
-        </is>
-      </c>
-      <c r="B91" t="inlineStr">
-        <is>
-          <t>emp_1781043065177</t>
-        </is>
-      </c>
-      <c r="C91" t="inlineStr">
-        <is>
-          <t>day_off</t>
-        </is>
-      </c>
-      <c r="D91" t="inlineStr">
-        <is>
-          <t>2026-06-12</t>
-        </is>
-      </c>
-      <c r="E91" t="inlineStr">
-        <is>
-          <t>2026-06-12</t>
-        </is>
-      </c>
-      <c r="F91" t="inlineStr">
-        <is>
-          <t>["saturday"]</t>
-        </is>
-      </c>
-      <c r="I91" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="K91" t="inlineStr">
-        <is>
-          <t>Have an external event.</t>
-        </is>
-      </c>
-      <c r="M91" s="463" t="n">
-        <v>46182.80686585648</v>
-      </c>
-      <c r="N91" s="463" t="n">
-        <v>46182.80738541667</v>
-      </c>
-      <c r="O91" t="inlineStr">
-        <is>
-          <t>emp_1780946033840</t>
-        </is>
-      </c>
-      <c r="P91" s="463" t="n">
-        <v>46182.80738541667</v>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" t="inlineStr">
-        <is>
-          <t>8b88681b-4d8c-4765-a0ed-34f658bc02ef</t>
-        </is>
-      </c>
-      <c r="B92" t="inlineStr">
-        <is>
-          <t>emp_1781047684821</t>
-        </is>
-      </c>
-      <c r="C92" t="inlineStr">
-        <is>
-          <t>day_off</t>
-        </is>
-      </c>
-      <c r="D92" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E92" t="inlineStr">
-        <is>
-          <t>2026-06-22</t>
-        </is>
-      </c>
-      <c r="F92" t="inlineStr">
-        <is>
-          <t>["monday"]</t>
-        </is>
-      </c>
-      <c r="I92" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="M92" s="463" t="n">
-        <v>46182.81649952546</v>
-      </c>
-      <c r="N92" s="463" t="n">
-        <v>46182.81891037037</v>
-      </c>
-      <c r="O92" t="inlineStr">
-        <is>
-          <t>emp_1780946033840</t>
-        </is>
-      </c>
-      <c r="P92" s="463" t="n">
-        <v>46182.81891037037</v>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" t="inlineStr">
-        <is>
-          <t>72d4bfe1-dd9b-402e-a50e-b348cf60a70f</t>
-        </is>
-      </c>
-      <c r="B93" t="inlineStr">
-        <is>
-          <t>emp_1781047684821</t>
-        </is>
-      </c>
-      <c r="C93" t="inlineStr">
-        <is>
-          <t>day_off</t>
-        </is>
-      </c>
-      <c r="D93" t="inlineStr">
-        <is>
-          <t>2026-06-17</t>
-        </is>
-      </c>
-      <c r="E93" t="inlineStr">
-        <is>
-          <t>2026-06-17</t>
-        </is>
-      </c>
-      <c r="F93" t="inlineStr">
-        <is>
-          <t>["thursday"]</t>
-        </is>
-      </c>
-      <c r="I93" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.REJECTED</t>
-        </is>
-      </c>
-      <c r="J93" t="inlineStr">
-        <is>
-          <t>Sorry.</t>
-        </is>
-      </c>
-      <c r="M93" s="463" t="n">
-        <v>46182.81661243056</v>
-      </c>
-      <c r="N93" s="463" t="n">
-        <v>46182.81902396991</v>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" t="inlineStr">
-        <is>
-          <t>d4aaa49b-72e3-4e1c-9db0-c68ab1ca966f</t>
-        </is>
-      </c>
-      <c r="B94" t="inlineStr">
-        <is>
-          <t>emp_1781047684821</t>
-        </is>
-      </c>
-      <c r="C94" t="inlineStr">
-        <is>
-          <t>day_off</t>
-        </is>
-      </c>
-      <c r="D94" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="E94" t="inlineStr">
-        <is>
-          <t>2026-06-23</t>
-        </is>
-      </c>
-      <c r="F94" t="inlineStr">
-        <is>
-          <t>["monday"]</t>
-        </is>
-      </c>
-      <c r="I94" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="M94" s="463" t="n">
-        <v>46182.82825238426</v>
-      </c>
-      <c r="N94" s="463" t="n">
-        <v>46182.83096163195</v>
-      </c>
-      <c r="O94" t="inlineStr">
-        <is>
-          <t>emp_1780946033840</t>
-        </is>
-      </c>
-      <c r="P94" s="463" t="n">
-        <v>46182.83096163195</v>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" t="inlineStr">
-        <is>
-          <t>365e0a5b-8b06-4ca7-a1c8-92c4eb3bd061</t>
-        </is>
-      </c>
-      <c r="B95" t="inlineStr">
-        <is>
-          <t>emp_1781047684821</t>
-        </is>
-      </c>
-      <c r="C95" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D95" t="inlineStr">
-        <is>
-          <t>2026-06-16</t>
-        </is>
-      </c>
-      <c r="E95" t="inlineStr">
-        <is>
-          <t>2026-06-23</t>
-        </is>
-      </c>
-      <c r="F95" t="inlineStr">
-        <is>
-          <t>["tuesday"]</t>
-        </is>
-      </c>
-      <c r="G95" t="inlineStr">
-        <is>
-          <t>09:00</t>
-        </is>
-      </c>
-      <c r="H95" t="inlineStr">
-        <is>
-          <t>12:00</t>
-        </is>
-      </c>
-      <c r="I95" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="M95" s="463" t="n">
-        <v>46182.82825482639</v>
-      </c>
-      <c r="N95" s="463" t="n">
-        <v>46182.83103702546</v>
-      </c>
-      <c r="O95" t="inlineStr">
-        <is>
-          <t>emp_1780946033840</t>
-        </is>
-      </c>
-      <c r="P95" s="463" t="n">
-        <v>46182.83103702546</v>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" t="inlineStr">
-        <is>
-          <t>db51084f-522f-4856-9371-22fcafe50cbf</t>
-        </is>
-      </c>
-      <c r="B96" t="inlineStr">
-        <is>
-          <t>emp_1781047684821</t>
-        </is>
-      </c>
-      <c r="C96" t="inlineStr">
-        <is>
-          <t>availability</t>
-        </is>
-      </c>
-      <c r="D96" t="inlineStr">
-        <is>
-          <t>2026-06-10</t>
-        </is>
-      </c>
-      <c r="E96" t="inlineStr">
-        <is>
-          <t>2026-06-24</t>
-        </is>
-      </c>
-      <c r="F96" t="inlineStr">
-        <is>
-          <t>["wednesday"]</t>
-        </is>
-      </c>
-      <c r="G96" t="inlineStr">
-        <is>
-          <t>09:00</t>
-        </is>
-      </c>
-      <c r="H96" t="inlineStr">
-        <is>
-          <t>15:00</t>
-        </is>
-      </c>
-      <c r="I96" t="inlineStr">
-        <is>
-          <t>AvailabilityRequestStatus.APPROVED</t>
-        </is>
-      </c>
-      <c r="M96" s="463" t="n">
-        <v>46182.83061645833</v>
-      </c>
-      <c r="N96" s="463" t="n">
-        <v>46182.83112265047</v>
-      </c>
-      <c r="O96" t="inlineStr">
-        <is>
-          <t>emp_1780946033840</t>
-        </is>
-      </c>
-      <c r="P96" s="463" t="n">
-        <v>46182.83112265047</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix day off shifts to not count toward total hours
</commit_message>
<xml_diff>
--- a/api/backend/uploads/ibu_schedule.xlsx
+++ b/api/backend/uploads/ibu_schedule.xlsx
@@ -62577,7 +62577,7 @@
         <v>46182.83089908565</v>
       </c>
       <c r="F189" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="190">
@@ -62605,7 +62605,7 @@
         <v>46182.83092059028</v>
       </c>
       <c r="F190" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="191">
@@ -62633,7 +62633,7 @@
         <v>46182.83095525463</v>
       </c>
       <c r="F191" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="192">
@@ -62661,7 +62661,7 @@
         <v>46182.83097667824</v>
       </c>
       <c r="F192" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="193">
@@ -62689,7 +62689,7 @@
         <v>46182.83103047454</v>
       </c>
       <c r="F193" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="194">
@@ -62717,7 +62717,7 @@
         <v>46182.83105209491</v>
       </c>
       <c r="F194" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="195">
@@ -62745,7 +62745,7 @@
         <v>46182.83111395833</v>
       </c>
       <c r="F195" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="196">
@@ -62773,7 +62773,7 @@
         <v>46182.83114960648</v>
       </c>
       <c r="F196" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix EmployeeUpdate model to accept string keys for preferences
</commit_message>
<xml_diff>
--- a/api/backend/uploads/ibu_schedule.xlsx
+++ b/api/backend/uploads/ibu_schedule.xlsx
@@ -57156,7 +57156,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:L3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -57268,6 +57268,50 @@
       </c>
       <c r="K2" s="463" t="n">
         <v>46182.68622203704</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>event_f48a0a04</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Party</t>
+        </is>
+      </c>
+      <c r="C3" s="462" t="n">
+        <v>46195</v>
+      </c>
+      <c r="D3" s="462" t="n">
+        <v>46184</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>22:00</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>ground floor</t>
+        </is>
+      </c>
+      <c r="H3" t="n">
+        <v>3</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>emp_1780946033840</t>
+        </is>
+      </c>
+      <c r="K3" s="463" t="n">
+        <v>46184.27980875</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Reset admin password to admin123
</commit_message>
<xml_diff>
--- a/api/backend/uploads/ibu_schedule.xlsx
+++ b/api/backend/uploads/ibu_schedule.xlsx
@@ -14447,7 +14447,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>888281da8992ec02</t>
+          <t>240be518fabd2724</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -14457,7 +14457,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-06-14T17:27:37.788767</t>
+          <t>2026-06-14T20:03:50.444560</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix admin password hash for admin123
</commit_message>
<xml_diff>
--- a/api/backend/uploads/ibu_schedule.xlsx
+++ b/api/backend/uploads/ibu_schedule.xlsx
@@ -503,7 +503,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
     <col width="40" customWidth="1" min="2" max="2"/>
@@ -587,7 +587,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N36"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -2449,7 +2449,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N30"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -4000,7 +4000,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N29"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -5495,7 +5495,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N34"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -7270,7 +7270,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N37"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -9173,7 +9173,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N22"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -10316,7 +10316,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N19"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -11326,7 +11326,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N15"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -12122,7 +12122,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N20"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -13163,7 +13163,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N24"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -14398,7 +14398,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
     <col width="25" customWidth="1" min="2" max="2"/>
@@ -14453,11 +14453,6 @@
       <c r="D2" t="inlineStr">
         <is>
           <t>manager</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>2026-06-14T20:03:50.444560</t>
         </is>
       </c>
     </row>
@@ -14473,7 +14468,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N20"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -15519,7 +15514,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N16"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -16361,7 +16356,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -17111,7 +17106,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N15"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -17897,7 +17892,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N25"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -19173,7 +19168,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N18"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -20107,7 +20102,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N19"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -21092,7 +21087,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N12"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -21745,7 +21740,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N15"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -22531,7 +22526,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N22"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -23639,7 +23634,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:H1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
@@ -23705,7 +23700,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N24"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -24900,7 +24895,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N35"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -26611,7 +26606,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N39"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -28531,7 +28526,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N36"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -30293,7 +30288,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N25"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -31519,7 +31514,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N21"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -32556,7 +32551,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -33266,7 +33261,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N41"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -35283,7 +35278,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N27"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -36641,7 +36636,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N34"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -38296,7 +38291,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:P1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -38410,7 +38405,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N40"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -40351,7 +40346,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N33"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -41955,7 +41950,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N27"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -43288,7 +43283,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N25"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -44504,7 +44499,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N25"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -45715,7 +45710,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N26"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -46972,7 +46967,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N20"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -47998,7 +47993,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N31"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -49485,7 +49480,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N21"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -50517,7 +50512,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N15"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -51308,7 +51303,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N26"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -52650,7 +52645,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N40"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -54691,7 +54686,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N51"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -57303,7 +57298,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N23"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>

</xml_diff>